<commit_message>
Update Western Canada internships spreadsheet 2026-04-02
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -476,7 +476,7 @@
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -535,7 +535,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://edel.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2001/job/22504</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://meredith.wd5.myworkdayjobs.com/en-US/EXT/job/Alberta-CAN-Remote/Data-Engineering-Intern_JR15360</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://semtech.wd1.myworkdayjobs.com/SemtechJobs/job/CAN---Richmond-BC/Software-Developer---Web-Cloud-Application--Co-op_REQ3167</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern-ML-AI/213550</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://revvity.wd103.myworkdayjobs.com/External/job/CAD-Remote--ON/Full-Stack-AI-Developer-Intern_JR-043679</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556851162</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---North-America/Software-Engineering-Intern--Cloud-Architecture_R-11509</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://meredith.wd5.myworkdayjobs.com/en-US/EXT/job/Alberta-CAN-Remote/Software-Engineering-Intern_JR15315-1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Innovation---Testing-Student--4-months----Summer-2026_JR157796</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Apparel-Design-Student--4-months----Summer-2026_JR157798-1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://emit.fa.ca3.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2001/job/82638</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://hdhl.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1004718</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.lever.co/kabam/0ffd4c22-8075-44a0-bb6d-4953219b3a49</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://job-boards.greenhouse.io/ada18/jobs/5063079007</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.lever.co/kabam/3e547642-cba0-43e3-8f7f-1b00b2befc13</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://job-boards.greenhouse.io/internshiplist2000/jobs/4998151008</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://careers.rivian.com/careers-home/jobs/28274</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://apply.workable.com/datavisor-jobs/j/2FB6A93BF6/</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27482</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Apply Here</t>
+          <t>https://jobs.lever.co/theathletic/e55c3738-517a-4033-843d-0c572f63145e</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -6030,36 +6030,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F194"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-04-05
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:F195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Diligent Corporation</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://edel.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2001/job/22504</t>
+          <t>https://job-boards.greenhouse.io/diligentcorporation/jobs/5834974004</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Mar 31, 2026</t>
+          <t>Apr 1, 2026</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Canadian Tire</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Software Developer. Web/Cloud Application</t>
+          <t>Apparel Design Student</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://semtech.wd1.myworkdayjobs.com/SemtechJobs/job/CAN---Richmond-BC/Software-Developer---Web-Cloud-Application--Co-op_REQ3167</t>
+          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Apparel-Design-Student--4-months----Summer-2026_JR157798-1</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mar 26, 2026</t>
+          <t>Mar 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern ML AI, Fall 2026</t>
+          <t>Health Informatics Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern-ML-AI/213550</t>
+          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mar 24, 2026</t>
+          <t>Mar 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Data Enablement</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://revvity.wd103.myworkdayjobs.com/External/job/CAD-Remote--ON/Full-Stack-AI-Developer-Intern_JR-043679</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mar 23, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer, The Coalition: Intern Opportunities</t>
+          <t>Safety Research Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556851162</t>
+          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Mar 20, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Cloud Architecture</t>
+          <t>User Research Co-op</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---North-America/Software-Engineering-Intern--Cloud-Architecture_R-11509</t>
+          <t>https://jobs.lever.co/kabam/0ffd4c22-8075-44a0-bb6d-4953219b3a49</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Feb 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>People Inc</t>
+          <t>Sanctuary AI</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,29 +759,29 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://meredith.wd5.myworkdayjobs.com/en-US/EXT/job/Alberta-CAN-Remote/Software-Engineering-Intern_JR15315-1</t>
+          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Canadian Tire</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Innovation &amp; Testing Student</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,29 +791,29 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Innovation---Testing-Student--4-months----Summer-2026_JR157796</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Canadian Tire</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Apparel Design Student</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -823,24 +823,24 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Apparel-Design-Student--4-months----Summer-2026_JR157798-1</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>WSP</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Web Developer Intern</t>
+          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://emit.fa.ca3.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2001/job/82638</t>
+          <t>https://careers.rivian.com/careers-home/jobs/28274</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Dec 12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>DataVisor</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Health Informatics Intern</t>
+          <t>Backend Software Engineer Internship</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
+          <t>https://apply.workable.com/datavisor-jobs/j/2FB6A93BF6/</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mar 10, 2026</t>
+          <t>Dec 10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Data Enablement</t>
+          <t>Software Engineering Intern – Connected Systems – Summer 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Safety Research Intern</t>
+          <t>Software Automation Engineering Intern – Summer 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,477 +951,425 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27482</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GIS Intern, Geospatial Services</t>
+          <t>Software Engineering Intern – Applications – Infotainment &amp; Mobile</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Nov 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Fortinet</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Product Management Intern</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Burnaby, BC</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Mar 31, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Semtech</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Software Developer. Web/Cloud Application</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Richmond, BC</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Mar 26, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern ML AI, Fall 2026</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Mar 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Full-Stack AI Developer Intern</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Mar 23, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer, The Coalition: Intern Opportunities</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Mar 20, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Calix</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern, Cloud Architecture</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Mar 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>DotDash Meredith</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Transaction Tooling Intern</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Mar 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer. Intern Opportunities for University Students</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Mar 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>People Inc</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Mar 13, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Canadian Tire</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Innovation &amp; Testing Student</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
           <t>Calgary, AB</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>https://hdhl.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1004718</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Mar 4, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Kabam</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>User Research Co-op</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/kabam/0ffd4c22-8075-44a0-bb6d-4953219b3a49</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Feb 26, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Ada</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Mar 13, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>WSP</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Web Developer Intern</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Mar 13, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Juniper Square</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/ada18/jobs/5063079007</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Feb 25, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Kabam</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer Co-op (Systems)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/kabam/3e547642-cba0-43e3-8f7f-1b00b2befc13</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Feb 24, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Sanctuary AI</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Feb 18, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Tenstorrent</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>IP Product Operations</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Feb 4, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Geotab</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Software Developer Intern - Echo</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Burnaby, BC</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/internshiplist2000/jobs/4998151008</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Dec 18</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/28274</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Dec 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>DataVisor</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Backend Software Engineer Internship</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>https://apply.workable.com/datavisor-jobs/j/2FB6A93BF6/</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Dec 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern – Connected Systems – Summer 2026</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Nov 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Software Automation Engineering Intern – Summer 2026</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27482</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Nov 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern – Applications – Infotainment &amp; Mobile</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Nov 5</t>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>The Athletic</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Engineering Student Intern, Summer 2026</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Remote in Canada</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/theathletic/e55c3738-517a-4033-843d-0c572f63145e</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Oct 17</t>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>AssetWorks</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Software Developer Intern</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>DotDash Meredith</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Transaction Tooling Intern</t>
+          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1432,24 +1380,24 @@
       <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer. Intern Opportunities for University Students</t>
+          <t>Software Engineering Intern, Data Engineer</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1460,24 +1408,24 @@
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Juniper Square</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer Intern</t>
+          <t>GIS Intern, Geospatial Services</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1488,24 +1436,24 @@
       <c r="E32" s="4" t="inlineStr"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Mar 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>AssetWorks</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Developer Co-op</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Waterloo, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1516,24 +1464,24 @@
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Mar 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
+          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1544,19 +1492,19 @@
       <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Data Engineer</t>
+          <t>Full-Stack Engineer Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1572,24 +1520,24 @@
       <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Developer Co-op</t>
+          <t>Frontend Engineering Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Waterloo, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1600,24 +1548,24 @@
       <c r="E36" s="4" t="inlineStr"/>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Mar 3, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1628,24 +1576,24 @@
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack Engineer Intern, Fall 2026</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1656,24 +1604,24 @@
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern, Fall 2026</t>
+          <t>Localization Software Developer, Co-Op</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1684,24 +1632,24 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1712,24 +1660,24 @@
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Correlation One</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1740,19 +1688,19 @@
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Localization Software Developer, Co-Op</t>
+          <t>Software Engineer Co-op (Systems)</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -1768,19 +1716,19 @@
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Correlation One</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
+          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -1796,19 +1744,19 @@
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>Jonas Software</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
+          <t>Jonas Summer Internship – Various Departments</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1831,17 +1779,17 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Critical Mass</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Development Intern</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1859,17 +1807,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Critical Mass</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Development Intern</t>
+          <t>Data Analytics &amp; Automation Development Student</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB / Acheson, AB</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1880,24 +1828,24 @@
       <c r="E46" s="4" t="inlineStr"/>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Feb 19, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Automation Development Student</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Acheson, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1915,12 +1863,12 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Automation Consulting Intern/Co-op</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -1936,24 +1884,24 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>CAE</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Automation Consulting Intern/Co-op</t>
+          <t>C-MAT-100 Engineering Intern</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Moose Jaw, SK</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1964,24 +1912,24 @@
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Feb 17, 2026</t>
+          <t>Feb 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>CAE</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>C-MAT-100 Engineering Intern</t>
+          <t>Application Engineer Test Intern</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Moose Jaw, SK</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1999,17 +1947,17 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>RSM</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Application Engineer Test Intern</t>
+          <t>Business Intelligence Consulting Associate - Fall 2026</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2020,24 +1968,24 @@
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Feb 16, 2026</t>
+          <t>Feb 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>RSM</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Business Intelligence Consulting Associate - Fall 2026</t>
+          <t>Student Digital Systems</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2048,24 +1996,24 @@
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Feb 13, 2026</t>
+          <t>Feb 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Student Digital Systems</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2076,24 +2024,24 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Feb 11, 2026</t>
+          <t>Feb 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Design Methodology Engineering Intern</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2116,7 +2064,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Design Methodology Engineering Intern</t>
+          <t>System Simulation Engineer Intern</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -2139,17 +2087,17 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Fullscript</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>System Simulation Engineer Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2167,17 +2115,17 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Fullscript</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Ottawa, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2188,19 +2136,19 @@
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Feb 10, 2026</t>
+          <t>Feb 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Applied Research Intern</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -2223,17 +2171,17 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Applied Research Intern</t>
+          <t>Intern, Dto, Enterprise Analytics</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2256,7 +2204,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Intern, Dto, Enterprise Analytics</t>
+          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -2284,7 +2232,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
+          <t>Intern, Data &amp; Integrations</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -2307,12 +2255,12 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Intern, Data &amp; Integrations</t>
+          <t>Design Validation Intern/Co-op</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -2335,17 +2283,17 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Mikata Health</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Design Validation Intern/Co-op</t>
+          <t>Healthcare Data Science Intern</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2363,17 +2311,17 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Mikata Health</t>
+          <t>Instacart</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Data Science Intern</t>
+          <t>Data Science PhD Intern</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2384,19 +2332,19 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Feb 9, 2026</t>
+          <t>Feb 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Instacart</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Data Science PhD Intern</t>
+          <t>Developer Intern - Client Secrets Management</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2412,24 +2360,24 @@
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Feb 5, 2026</t>
+          <t>Feb 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Client Secrets Management</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2440,24 +2388,24 @@
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Feb 3, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Data Intern - Enterprise Analytics</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2475,17 +2423,17 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Veralto</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Data Intern - Enterprise Analytics</t>
+          <t>Machine Learning Co-Op Intern</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2496,24 +2444,24 @@
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Feb 2, 2026</t>
+          <t>Feb 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Veralto</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Co-Op Intern</t>
+          <t>Developer Intern - Knox</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2524,7 +2472,7 @@
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Feb 1, 2026</t>
+          <t>Jan 30, 2026</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2484,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Knox</t>
+          <t>Developer Intern - Trust Platforms</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -2564,7 +2512,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Trust Platforms</t>
+          <t>Developer Intern - Extension Excellence</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -2592,7 +2540,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Extension Excellence</t>
+          <t>Developer Intern - Insights</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -2620,7 +2568,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Insights</t>
+          <t>Developer Intern - Platform Advancement</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -2648,7 +2596,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement</t>
+          <t>Developer Intern - Device Security</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -2676,7 +2624,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Device Security</t>
+          <t>Developer Intern - Billing &amp; Payments</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -2704,7 +2652,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Billing &amp; Payments</t>
+          <t>Developer Intern - Data &amp; Access</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -2727,17 +2675,17 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Data &amp; Access</t>
+          <t>Student Engineer</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2755,17 +2703,17 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>Voldex</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Student Engineer</t>
+          <t>Game Developer Intern</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2776,19 +2724,19 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Jan 30, 2026</t>
+          <t>Jan 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Voldex</t>
+          <t>GE Healthcare</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Game Developer Intern</t>
+          <t>Field Service Apprentice</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -2804,24 +2752,24 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Jan 29, 2026</t>
+          <t>Jan 28, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>GE Healthcare</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Field Service Apprentice</t>
+          <t>Software Engineer Co-Op</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2839,17 +2787,17 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-Op</t>
+          <t>Software Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2860,24 +2808,24 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Jan 28, 2026</t>
+          <t>Jan 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>BC Pensions</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern/Co-op</t>
+          <t>Application Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2895,17 +2843,17 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>BC Pensions</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Application Developer Intern/Co-op</t>
+          <t>Support Enablement Engineer Intern</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2916,19 +2864,19 @@
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Jan 26, 2026</t>
+          <t>Jan 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Support Enablement Engineer Intern</t>
+          <t>Intern Full Stack Developer</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -2951,12 +2899,12 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Allstate Insurance Company</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Intern Full Stack Developer</t>
+          <t>Data Governance Intern/Co-op</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2972,7 +2920,7 @@
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Jan 23, 2026</t>
+          <t>Jan 22, 2026</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2932,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Data Governance Intern/Co-op</t>
+          <t>Provincial Product Analyst Co-op</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -3007,17 +2955,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Allstate Insurance Company</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Provincial Product Analyst Co-op</t>
+          <t>Production Engineering Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3028,7 +2976,7 @@
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Jan 22, 2026</t>
+          <t>Jan 21, 2026</t>
         </is>
       </c>
     </row>
@@ -3040,7 +2988,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern - Summer 2026</t>
+          <t>Studio Talent Group Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -3068,7 +3016,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern - Summer 2026</t>
+          <t>Graduate Production Engineer Research Intern</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -3096,7 +3044,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Graduate Production Engineer Research Intern</t>
+          <t>Technical Assistant Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -3119,17 +3067,17 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>BMO</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Technical Assistant Intern - Summer 2026</t>
+          <t>Software Developer – Co-op/Internship</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3140,19 +3088,19 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Jan 21, 2026</t>
+          <t>Jan 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>BMO</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Co-op/Internship</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -3175,17 +3123,17 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>Boomi</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Engineering Intern</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3196,24 +3144,24 @@
       <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Jan 19, 2026</t>
+          <t>Jan 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>The Boeing Company</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Engineering Intern</t>
+          <t>Data Engineering Intern</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -3224,7 +3172,7 @@
       <c r="E94" s="4" t="inlineStr"/>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Jan 17, 2026</t>
+          <t>Jan 16, 2026</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3184,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -3264,7 +3212,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Data Science Business Operations Intern</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -3287,17 +3235,17 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>The Boeing Company</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Data Science Business Operations Intern</t>
+          <t>Systems Analyst</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3315,12 +3263,12 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Systems Analyst</t>
+          <t>AI/ML Coop/Intern</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -3343,17 +3291,17 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Enbridge</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>AI/ML Coop/Intern</t>
+          <t>SharePoint &amp; Document Management Support - Summer Student</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3371,17 +3319,17 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Enbridge</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>SharePoint &amp; Document Management Support - Summer Student</t>
+          <t>Game Creation SW Engineer Intern</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -3392,24 +3340,24 @@
       <c r="E100" s="4" t="inlineStr"/>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Jan 16, 2026</t>
+          <t>Jan 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Game Creation SW Engineer Intern</t>
+          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3432,7 +3380,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -3455,17 +3403,17 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3476,19 +3424,19 @@
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Jan 15, 2026</t>
+          <t>Jan 13</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer - Internship Opportunities</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -3504,24 +3452,24 @@
       <c r="E104" s="4" t="inlineStr"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Jan 13</t>
+          <t>Jan 12</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer - Internship Opportunities</t>
+          <t>Systems Software Engineering Intern</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote in Canada</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -3532,24 +3480,24 @@
       <c r="E105" s="4" t="inlineStr"/>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Jan 12</t>
+          <t>Jan 9</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineering Intern</t>
+          <t>Triton Compiler Engineering Intern</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote in Canada</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -3567,17 +3515,17 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Triton Compiler Engineering Intern</t>
+          <t>Software Developer - Co-op - Full Stack</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -3600,7 +3548,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - Co-op - Full Stack</t>
+          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -3628,7 +3576,7 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
+          <t>Software Developer - C++ - Co-op</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -3651,12 +3599,12 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - C++ - Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -3679,17 +3627,17 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -3700,24 +3648,24 @@
       <c r="E111" s="4" t="inlineStr"/>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>Jan 9</t>
+          <t>Jan 8</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op/Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -3735,7 +3683,7 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
@@ -3756,14 +3704,14 @@
       <c r="E113" s="4" t="inlineStr"/>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>Jan 8</t>
+          <t>Jan 7</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -3784,24 +3732,24 @@
       <c r="E114" s="4" t="inlineStr"/>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Jan 7</t>
+          <t>Jan 6</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Intern/Co-op - Oracle APEX</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -3812,24 +3760,24 @@
       <c r="E115" s="4" t="inlineStr"/>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Jan 6</t>
+          <t>Jan 5</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern/Co-op - Oracle APEX</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3847,17 +3795,17 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>BDC</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3875,17 +3823,17 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>BDC</t>
+          <t>Accenture</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
+          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
+          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -3896,7 +3844,7 @@
       <c r="E118" s="4" t="inlineStr"/>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Jan 5</t>
+          <t>Dec 20</t>
         </is>
       </c>
     </row>
@@ -3908,12 +3856,12 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
+          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -3931,17 +3879,17 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
+          <t>Software Developer Intern - Echo</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -3952,7 +3900,7 @@
       <c r="E120" s="4" t="inlineStr"/>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>Dec 20</t>
+          <t>Dec 18</t>
         </is>
       </c>
     </row>
@@ -4911,17 +4859,17 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>The Athletic</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>SAP Analytics Cloud Security Engineer Intern</t>
+          <t>Engineering Student Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
@@ -4932,24 +4880,24 @@
       <c r="E155" s="4" t="inlineStr"/>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>Oct 16</t>
+          <t>Oct 17</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>Journal Technologies</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Junior Software Developer Co-op</t>
+          <t>SAP Analytics Cloud Security Engineer Intern</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
@@ -4967,17 +4915,17 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Canada Life</t>
+          <t>Journal Technologies</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Student Position)</t>
+          <t>Junior Software Developer Co-op</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Winnipeg, MB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -4988,24 +4936,24 @@
       <c r="E157" s="4" t="inlineStr"/>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>Oct 15</t>
+          <t>Oct 16</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Canada Life</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Full-stack Engineering Intern</t>
+          <t>Software Developer (Student Position)</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Winnipeg, MB</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
@@ -5016,7 +4964,7 @@
       <c r="E158" s="4" t="inlineStr"/>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 15</t>
         </is>
       </c>
     </row>
@@ -5028,7 +4976,7 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Backend Engineering Intern</t>
+          <t>Full-stack Engineering Intern</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -5056,7 +5004,7 @@
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern</t>
+          <t>Backend Engineering Intern</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -5079,17 +5027,17 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern</t>
+          <t>Frontend Engineering Intern</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
@@ -5100,19 +5048,19 @@
       <c r="E161" s="4" t="inlineStr"/>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>Oct 10</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Intern – Digital Ship</t>
+          <t>Software Development Intern</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
@@ -5128,24 +5076,24 @@
       <c r="E162" s="4" t="inlineStr"/>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>Oct 8</t>
+          <t>Oct 10</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Intern – Digital Ship</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
@@ -5156,24 +5104,24 @@
       <c r="E163" s="4" t="inlineStr"/>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>Oct 7</t>
+          <t>Oct 8</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – Sports Technology</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
@@ -5184,7 +5132,7 @@
       <c r="E164" s="4" t="inlineStr"/>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 7</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5144,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – UFC</t>
+          <t>Software Engineer Intern – Sports Technology</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -5219,17 +5167,17 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Stateful Systems - Winter 2026</t>
+          <t>Software Engineer Intern – UFC</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
@@ -5240,7 +5188,7 @@
       <c r="E166" s="4" t="inlineStr"/>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 6</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5200,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Release Engineering - Winter 2026</t>
+          <t>Developer Intern - Stateful Systems - Winter 2026</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -5280,7 +5228,7 @@
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement - Winter 2026</t>
+          <t>Developer Intern - Release Engineering - Winter 2026</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
@@ -5308,7 +5256,7 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Frameworks - Winter 2026</t>
+          <t>Developer Intern - Platform Advancement - Winter 2026</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -5336,7 +5284,7 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
+          <t>Developer Intern - Frameworks - Winter 2026</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -5364,7 +5312,7 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - App Launcher - Winter 2026</t>
+          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -5387,17 +5335,17 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Online Software Engineer Co-op</t>
+          <t>Developer Intern - App Launcher - Winter 2026</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
@@ -5408,24 +5356,24 @@
       <c r="E172" s="4" t="inlineStr"/>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Winter 2026</t>
+          <t>Online Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
@@ -5436,24 +5384,24 @@
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 4</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
+          <t>Software Development Engineer Internship – Winter 2026</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -5464,7 +5412,7 @@
       <c r="E174" s="4" t="inlineStr"/>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 3</t>
         </is>
       </c>
     </row>
@@ -5476,7 +5424,7 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – NHL</t>
+          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -5504,7 +5452,7 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
+          <t>Software Engineer Intern – NHL</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
@@ -5527,12 +5475,12 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Front-end Co-Op</t>
+          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -5548,24 +5496,24 @@
       <c r="E177" s="4" t="inlineStr"/>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>Oct 1</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern – Multiple Teams</t>
+          <t>Software Developer – Front-end Co-Op</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
@@ -5576,24 +5524,24 @@
       <c r="E178" s="4" t="inlineStr"/>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>Sep 23</t>
+          <t>Oct 1</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Datahub)</t>
+          <t>Software Development Intern – Multiple Teams</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
@@ -5604,7 +5552,7 @@
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Sep 23</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5564,7 @@
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Quality Assurance)</t>
+          <t>Software Developer Intern (Datahub)</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
@@ -5644,7 +5592,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Enterprise Applications)</t>
+          <t>Software Developer Intern (Quality Assurance)</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -5667,12 +5615,12 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern/ Co-op</t>
+          <t>Software Developer Intern (Enterprise Applications)</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
@@ -5695,17 +5643,17 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Hewlett Packard (HP)</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Associate C++ Software Developer</t>
+          <t>Software Engineering Intern/ Co-op</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
@@ -5716,7 +5664,7 @@
       <c r="E183" s="4" t="inlineStr"/>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Sep 15</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
@@ -5751,17 +5699,17 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Hewlett Packard (HP)</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Intern – Software Developer</t>
+          <t>Associate C++ Software Developer</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
@@ -5772,24 +5720,24 @@
       <c r="E185" s="4" t="inlineStr"/>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>Sep 10</t>
+          <t>Sep 15</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Student</t>
+          <t>Intern – Software Developer</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
@@ -5800,24 +5748,24 @@
       <c r="E186" s="4" t="inlineStr"/>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>Sep 08</t>
+          <t>Sep 10</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer Co-op Student</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
@@ -5828,24 +5776,24 @@
       <c r="E187" s="4" t="inlineStr"/>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>Sep 05</t>
+          <t>Sep 08</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer: Internship Opportunities</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
@@ -5856,19 +5804,19 @@
       <c r="E188" s="4" t="inlineStr"/>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>Sep 5</t>
+          <t>Sep 05</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>Epic Games</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce Programmer Intern</t>
+          <t>Software Engineer: Internship Opportunities</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -5884,19 +5832,19 @@
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>Sep 04</t>
+          <t>Sep 5</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Epic Games</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Ecommerce Programmer Intern</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -5912,24 +5860,24 @@
       <c r="E190" s="4" t="inlineStr"/>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>Sep 01</t>
+          <t>Sep 04</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>TC Energy</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Computer Science Interns</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
@@ -5940,24 +5888,24 @@
       <c r="E191" s="4" t="inlineStr"/>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 01</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>Corpay</t>
+          <t>TC Energy</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Co-op)</t>
+          <t>Computer Science Interns</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
@@ -5968,24 +5916,24 @@
       <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Aug 31</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Corpay</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer (Co-op)</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
@@ -5996,19 +5944,19 @@
       <c r="E193" s="4" t="inlineStr"/>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>Aug 25</t>
+          <t>Aug 27</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -6024,12 +5972,40 @@
       <c r="E194" s="4" t="inlineStr"/>
       <c r="F194" s="4" t="inlineStr">
         <is>
+          <t>Aug 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Software</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Summer Internship – Various Departments</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>Remote in Canada</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr"/>
+      <c r="F195" s="4" t="inlineStr">
+        <is>
           <t>Aug 02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F194"/>
+  <autoFilter ref="A1:F195"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-04-26
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F207"/>
+  <dimension ref="A1:F208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -611,12 +611,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Revvity</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Test and Manufacturing Intern</t>
+          <t>Full-Stack AI Developer Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
+          <t>https://revvity.wd103.myworkdayjobs.com/External/job/CAD-Remote--ON/Full-Stack-AI-Developer-Intern_JR-044247</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Apr 16, 2026</t>
+          <t>Apr 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>OpusClip</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager Intern</t>
+          <t>Test and Manufacturing Intern</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
+          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Apr 14, 2026</t>
+          <t>Apr 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>OpusClip</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern</t>
+          <t>AI Product Manager Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Product-Management-Intern/210908</t>
+          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Apr 11, 2026</t>
+          <t>Apr 14, 2026</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>AI / Machine Learning Intern</t>
+          <t>Health Informatics Intern</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---North-America/AI---Machine-Learning-Intern_R-11566</t>
+          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apr 7, 2026</t>
+          <t>Mar 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Diligent Corporation</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Data Enablement</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/diligentcorporation/jobs/5834974004</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apr 1, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DotDash Meredith</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Safety Research Intern</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Remote</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://meredith.wd5.myworkdayjobs.com/en-US/EXT/job/Alberta-CAN-Remote/Data-Engineering-Intern_JR15360</t>
+          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Mar 31, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Canadian Tire</t>
+          <t>Sanctuary AI</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Apparel Design Student</t>
+          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,24 +983,24 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://canadiantirecorporation.wd3.myworkdayjobs.com/Enterprise_External_Careers_Site/job/Calgary-AB/Apparel-Design-Student--4-months----Summer-2026_JR157798-1</t>
+          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Health Informatics Intern</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1015,29 +1015,29 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Mar 10, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Data Enablement</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Safety Research Intern</t>
+          <t>Software Engineering Intern, Connected Systems, Summer 2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,24 +1079,24 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Sanctuary AI</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
+          <t>Software Engineering Intern – Applications – Infotainment &amp; Mobile</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1111,253 +1111,225 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
+          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Tenstorrent</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>IP Product Operations</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Product Management Intern</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Apr 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Calix</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>AI / Machine Learning Intern</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Feb 4, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Apr 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/28274</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Dec 12</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Diligent Corporation</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Apr 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>DataVisor</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Backend Software Engineer Internship</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>https://apply.workable.com/datavisor-jobs/j/2FB6A93BF6/</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Dec 10</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Fortinet</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Product Management Intern</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Burnaby, BC</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Mar 31, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern – Connected Systems – Summer 2026</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Nov 13</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>DotDash Meredith</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Data Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Remote</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Mar 31, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Software Automation Engineering Intern – Summer 2026</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27482</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Nov 13</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Semtech</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Software Developer. Web/Cloud Application</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Richmond, BC</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Mar 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern – Applications – Infotainment &amp; Mobile</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Nov 5</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern ML AI, Fall 2026</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Mar 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Revvity</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Product Management Intern</t>
+          <t>Full-Stack AI Developer Intern</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1368,24 +1340,24 @@
       <c r="E28" s="4" t="inlineStr"/>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Mar 31, 2026</t>
+          <t>Mar 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Software Developer. Web/Cloud Application</t>
+          <t>Software Engineer, The Coalition: Intern Opportunities</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1396,24 +1368,24 @@
       <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Mar 26, 2026</t>
+          <t>Mar 20, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern ML AI, Fall 2026</t>
+          <t>Software Engineering Intern, Cloud Architecture</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1424,24 +1396,24 @@
       <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Mar 24, 2026</t>
+          <t>Mar 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>DotDash Meredith</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Transaction Tooling Intern</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1452,7 +1424,7 @@
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Mar 23, 2026</t>
+          <t>Mar 18, 2026</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1436,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer, The Coalition: Intern Opportunities</t>
+          <t>Software Engineer. Intern Opportunities for University Students</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1480,19 +1452,19 @@
       <c r="E32" s="4" t="inlineStr"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Mar 20, 2026</t>
+          <t>Mar 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>People Inc</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Cloud Architecture</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1508,24 +1480,24 @@
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>DotDash Meredith</t>
+          <t>Canadian Tire</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Transaction Tooling Intern</t>
+          <t>Innovation &amp; Testing Student</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1536,24 +1508,24 @@
       <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Canadian Tire</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer. Intern Opportunities for University Students</t>
+          <t>Apparel Design Student</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1564,24 +1536,24 @@
       <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>People Inc</t>
+          <t>WSP</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Web Developer Intern</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1599,17 +1571,17 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Canadian Tire</t>
+          <t>Juniper Square</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Innovation &amp; Testing Student</t>
+          <t>AI Engineer Intern</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1620,24 +1592,24 @@
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>WSP</t>
+          <t>AssetWorks</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Web Developer Intern</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1648,24 +1620,24 @@
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Juniper Square</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer Intern</t>
+          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1676,24 +1648,24 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>AssetWorks</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Software Engineering Intern, Data Engineer</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1704,24 +1676,24 @@
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
+          <t>GIS Intern, Geospatial Services</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1732,24 +1704,24 @@
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Data Engineer</t>
+          <t>Developer Co-op</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Waterloo, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1760,24 +1732,24 @@
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>GIS Intern, Geospatial Services</t>
+          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1788,24 +1760,24 @@
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Mar 4, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Developer Co-op</t>
+          <t>Full-Stack Engineer Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Waterloo, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1816,7 +1788,7 @@
       <c r="E44" s="4" t="inlineStr"/>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Mar 3, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1800,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
+          <t>Frontend Engineering Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -1851,17 +1823,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack Engineer Intern, Fall 2026</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1872,24 +1844,24 @@
       <c r="E46" s="4" t="inlineStr"/>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern, Fall 2026</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1900,19 +1872,19 @@
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>User Research Co-op</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -1928,24 +1900,24 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Feb 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>Localization Software Developer, Co-Op</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1956,24 +1928,24 @@
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>User Research Co-op</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1984,24 +1956,24 @@
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Feb 26, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Correlation One</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Localization Software Developer, Co-Op</t>
+          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2019,17 +1991,17 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Software Engineer Co-op (Systems)</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2040,19 +2012,19 @@
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Correlation One</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
+          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -2068,24 +2040,24 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Jonas Software</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op (Systems)</t>
+          <t>Jonas Summer Internship – Various Departments</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2096,24 +2068,24 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Feb 24, 2026</t>
+          <t>Feb 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>Critical Mass</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
+          <t>Development Intern</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2131,17 +2103,17 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Data Analytics &amp; Automation Development Student</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB / Acheson, AB</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2152,24 +2124,24 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Feb 19, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Critical Mass</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Development Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2180,24 +2152,24 @@
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Feb 19, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Automation Development Student</t>
+          <t>Automation Consulting Intern/Co-op</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Acheson, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2208,24 +2180,24 @@
       <c r="E58" s="4" t="inlineStr"/>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>CAE</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>C-MAT-100 Engineering Intern</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Moose Jaw, SK</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2236,24 +2208,24 @@
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Automation Consulting Intern/Co-op</t>
+          <t>Application Engineer Test Intern</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2264,24 +2236,24 @@
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Feb 17, 2026</t>
+          <t>Feb 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>CAE</t>
+          <t>RSM</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>C-MAT-100 Engineering Intern</t>
+          <t>Business Intelligence Consulting Associate - Fall 2026</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Moose Jaw, SK</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2292,19 +2264,19 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Feb 16, 2026</t>
+          <t>Feb 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Application Engineer Test Intern</t>
+          <t>Student Digital Systems</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -2320,24 +2292,24 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Feb 16, 2026</t>
+          <t>Feb 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>RSM</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Business Intelligence Consulting Associate - Fall 2026</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2348,24 +2320,24 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Feb 13, 2026</t>
+          <t>Feb 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Student Digital Systems</t>
+          <t>Design Methodology Engineering Intern</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2376,24 +2348,24 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Feb 11, 2026</t>
+          <t>Feb 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>System Simulation Engineer Intern</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2411,17 +2383,17 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Fullscript</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Design Methodology Engineering Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2439,12 +2411,12 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>System Simulation Engineer Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -2460,24 +2432,24 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Feb 10, 2026</t>
+          <t>Feb 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Fullscript</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Applied Research Intern</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Ottawa, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2488,24 +2460,24 @@
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Feb 10, 2026</t>
+          <t>Feb 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Intern, Dto, Enterprise Analytics</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2523,17 +2495,17 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Applied Research Intern</t>
+          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2556,7 +2528,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Intern, Dto, Enterprise Analytics</t>
+          <t>Intern, Data &amp; Integrations</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -2579,12 +2551,12 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
+          <t>Design Validation Intern/Co-op</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -2607,17 +2579,17 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Mikata Health</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Intern, Data &amp; Integrations</t>
+          <t>Healthcare Data Science Intern</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2635,17 +2607,17 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Instacart</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Design Validation Intern/Co-op</t>
+          <t>Data Science PhD Intern</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2656,24 +2628,24 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Feb 9, 2026</t>
+          <t>Feb 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Mikata Health</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Data Science Intern</t>
+          <t>Developer Intern - Client Secrets Management</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2684,24 +2656,24 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Feb 9, 2026</t>
+          <t>Feb 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Instacart</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Data Science PhD Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2712,7 +2684,7 @@
       <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Feb 5, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2696,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Client Secrets Management</t>
+          <t>Data Intern - Enterprise Analytics</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -2740,24 +2712,24 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Feb 3, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>Veralto</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Machine Learning Co-Op Intern</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2768,7 +2740,7 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Feb 2, 2026</t>
+          <t>Feb 1, 2026</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2752,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Data Intern - Enterprise Analytics</t>
+          <t>Developer Intern - Knox</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -2796,24 +2768,24 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Feb 2, 2026</t>
+          <t>Jan 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Veralto</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Co-Op Intern</t>
+          <t>Developer Intern - Trust Platforms</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2824,7 +2796,7 @@
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Feb 1, 2026</t>
+          <t>Jan 30, 2026</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2808,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Knox</t>
+          <t>Developer Intern - Extension Excellence</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -2864,7 +2836,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Trust Platforms</t>
+          <t>Developer Intern - Insights</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -2892,7 +2864,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Extension Excellence</t>
+          <t>Developer Intern - Platform Advancement</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -2920,7 +2892,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Insights</t>
+          <t>Developer Intern - Device Security</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -2948,7 +2920,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement</t>
+          <t>Developer Intern - Billing &amp; Payments</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2976,7 +2948,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Device Security</t>
+          <t>Developer Intern - Data &amp; Access</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -2999,17 +2971,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Billing &amp; Payments</t>
+          <t>Student Engineer</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3027,12 +2999,12 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Voldex</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Data &amp; Access</t>
+          <t>Game Developer Intern</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -3048,24 +3020,24 @@
       <c r="E88" s="4" t="inlineStr"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Jan 30, 2026</t>
+          <t>Jan 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>GE Healthcare</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Student Engineer</t>
+          <t>Field Service Apprentice</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3076,24 +3048,24 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Jan 30, 2026</t>
+          <t>Jan 28, 2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Voldex</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Game Developer Intern</t>
+          <t>Software Engineer Co-Op</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3104,24 +3076,24 @@
       <c r="E90" s="4" t="inlineStr"/>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Jan 29, 2026</t>
+          <t>Jan 28, 2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>GE Healthcare</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Field Service Apprentice</t>
+          <t>Software Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3132,19 +3104,19 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Jan 28, 2026</t>
+          <t>Jan 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>BC Pensions</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-Op</t>
+          <t>Application Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -3160,24 +3132,24 @@
       <c r="E92" s="4" t="inlineStr"/>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Jan 28, 2026</t>
+          <t>Jan 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern/Co-op</t>
+          <t>Support Enablement Engineer Intern</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3188,24 +3160,24 @@
       <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Jan 26, 2026</t>
+          <t>Jan 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>BC Pensions</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Application Developer Intern/Co-op</t>
+          <t>Intern Full Stack Developer</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -3216,19 +3188,19 @@
       <c r="E94" s="4" t="inlineStr"/>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Jan 26, 2026</t>
+          <t>Jan 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Allstate Insurance Company</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Support Enablement Engineer Intern</t>
+          <t>Data Governance Intern/Co-op</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -3244,19 +3216,19 @@
       <c r="E95" s="4" t="inlineStr"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Jan 23, 2026</t>
+          <t>Jan 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Allstate Insurance Company</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Intern Full Stack Developer</t>
+          <t>Provincial Product Analyst Co-op</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -3272,24 +3244,24 @@
       <c r="E96" s="4" t="inlineStr"/>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Jan 23, 2026</t>
+          <t>Jan 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Allstate Insurance Company</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Data Governance Intern/Co-op</t>
+          <t>Production Engineering Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3300,24 +3272,24 @@
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Jan 22, 2026</t>
+          <t>Jan 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Allstate Insurance Company</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Provincial Product Analyst Co-op</t>
+          <t>Studio Talent Group Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -3328,7 +3300,7 @@
       <c r="E98" s="4" t="inlineStr"/>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Jan 22, 2026</t>
+          <t>Jan 21, 2026</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3312,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern - Summer 2026</t>
+          <t>Graduate Production Engineer Research Intern</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -3368,7 +3340,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern - Summer 2026</t>
+          <t>Technical Assistant Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -3391,17 +3363,17 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>BMO</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Graduate Production Engineer Research Intern</t>
+          <t>Software Developer – Co-op/Internship</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3412,24 +3384,24 @@
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Jan 21, 2026</t>
+          <t>Jan 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Technical Assistant Intern - Summer 2026</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -3440,24 +3412,24 @@
       <c r="E102" s="4" t="inlineStr"/>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Jan 21, 2026</t>
+          <t>Jan 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>BMO</t>
+          <t>Boomi</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Co-op/Internship</t>
+          <t>Engineering Intern</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3468,24 +3440,24 @@
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Jan 19, 2026</t>
+          <t>Jan 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>The Boeing Company</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Data Engineering Intern</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -3496,24 +3468,24 @@
       <c r="E104" s="4" t="inlineStr"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Jan 19, 2026</t>
+          <t>Jan 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>The Boeing Company</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Engineering Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -3524,7 +3496,7 @@
       <c r="E105" s="4" t="inlineStr"/>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Jan 17, 2026</t>
+          <t>Jan 16, 2026</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3508,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Data Science Business Operations Intern</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -3559,17 +3531,17 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>The Boeing Company</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Systems Analyst</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -3587,17 +3559,17 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>The Boeing Company</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Data Science Business Operations Intern</t>
+          <t>AI/ML Coop/Intern</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -3615,17 +3587,17 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>Enbridge</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Systems Analyst</t>
+          <t>SharePoint &amp; Document Management Support - Summer Student</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -3643,17 +3615,17 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>AI/ML Coop/Intern</t>
+          <t>Game Creation SW Engineer Intern</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -3664,24 +3636,24 @@
       <c r="E110" s="4" t="inlineStr"/>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>Jan 16, 2026</t>
+          <t>Jan 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Enbridge</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>SharePoint &amp; Document Management Support - Summer Student</t>
+          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -3692,24 +3664,24 @@
       <c r="E111" s="4" t="inlineStr"/>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>Jan 16, 2026</t>
+          <t>Jan 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Game Creation SW Engineer Intern</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -3727,17 +3699,17 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -3748,24 +3720,24 @@
       <c r="E113" s="4" t="inlineStr"/>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>Jan 15, 2026</t>
+          <t>Jan 13</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Software Engineer - Internship Opportunities</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -3776,24 +3748,24 @@
       <c r="E114" s="4" t="inlineStr"/>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Jan 15, 2026</t>
+          <t>Jan 12</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Systems Software Engineering Intern</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote in Canada</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -3804,24 +3776,24 @@
       <c r="E115" s="4" t="inlineStr"/>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Jan 13</t>
+          <t>Jan 9</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer - Internship Opportunities</t>
+          <t>Triton Compiler Engineering Intern</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3832,24 +3804,24 @@
       <c r="E116" s="4" t="inlineStr"/>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>Jan 12</t>
+          <t>Jan 9</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineering Intern</t>
+          <t>Software Developer - Co-op - Full Stack</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3867,17 +3839,17 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Triton Compiler Engineering Intern</t>
+          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -3900,7 +3872,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - Co-op - Full Stack</t>
+          <t>Software Developer - C++ - Co-op</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -3923,12 +3895,12 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
@@ -3951,17 +3923,17 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - C++ - Co-op</t>
+          <t>Software Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -3972,19 +3944,19 @@
       <c r="E121" s="4" t="inlineStr"/>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>Jan 9</t>
+          <t>Jan 8</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
@@ -4000,24 +3972,24 @@
       <c r="E122" s="4" t="inlineStr"/>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>Jan 9</t>
+          <t>Jan 8</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op/Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -4028,7 +4000,7 @@
       <c r="E123" s="4" t="inlineStr"/>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>Jan 8</t>
+          <t>Jan 7</t>
         </is>
       </c>
     </row>
@@ -4056,24 +4028,24 @@
       <c r="E124" s="4" t="inlineStr"/>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>Jan 8</t>
+          <t>Jan 6</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Intern/Co-op - Oracle APEX</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -4084,14 +4056,14 @@
       <c r="E125" s="4" t="inlineStr"/>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>Jan 7</t>
+          <t>Jan 5</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -4112,24 +4084,24 @@
       <c r="E126" s="4" t="inlineStr"/>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>Jan 6</t>
+          <t>Jan 5</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>BDC</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern/Co-op - Oracle APEX</t>
+          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -4147,17 +4119,17 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Accenture</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -4168,24 +4140,24 @@
       <c r="E128" s="4" t="inlineStr"/>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>Jan 5</t>
+          <t>Dec 20</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>BDC</t>
+          <t>Accenture</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
+          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
+          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -4196,24 +4168,24 @@
       <c r="E129" s="4" t="inlineStr"/>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>Jan 5</t>
+          <t>Dec 20</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
+          <t>Software Developer Intern - Echo</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -4224,24 +4196,24 @@
       <c r="E130" s="4" t="inlineStr"/>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>Dec 20</t>
+          <t>Dec 18</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -4252,24 +4224,24 @@
       <c r="E131" s="4" t="inlineStr"/>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>Dec 20</t>
+          <t>Dec 17</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern - Echo</t>
+          <t>Software Engineer Intern - AI/ML QVS</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -4280,24 +4252,24 @@
       <c r="E132" s="4" t="inlineStr"/>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>Dec 18</t>
+          <t>Dec 15</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>RBC Borealis - Machine Learning Software Engineer</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -4308,19 +4280,19 @@
       <c r="E133" s="4" t="inlineStr"/>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>Dec 17</t>
+          <t>Dec 12</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - AI/ML QVS</t>
+          <t>Software Engineering Intern, Applications - Summer 2026</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
@@ -4336,24 +4308,24 @@
       <c r="E134" s="4" t="inlineStr"/>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>Dec 15</t>
+          <t>Dec 12</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>RBC Borealis - Machine Learning Software Engineer</t>
+          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -4371,12 +4343,12 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Applications - Summer 2026</t>
+          <t>Production Engineering Intern</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
@@ -4404,7 +4376,7 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern</t>
+          <t>Studio Talent Group Intern</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -4420,19 +4392,19 @@
       <c r="E137" s="4" t="inlineStr"/>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>Dec 12</t>
+          <t>Dec 11</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>DataVisor</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern</t>
+          <t>Backend Software Engineer Internship</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
@@ -4448,7 +4420,7 @@
       <c r="E138" s="4" t="inlineStr"/>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>Dec 11</t>
+          <t>Dec 10</t>
         </is>
       </c>
     </row>
@@ -4651,12 +4623,12 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>Transcarent</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Software Engineer Intern</t>
+          <t>Software Automation Engineering Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
@@ -4672,24 +4644,24 @@
       <c r="E146" s="4" t="inlineStr"/>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>Nov 7</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>Valsoft Corporation</t>
+          <t>Transcarent</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
+          <t>Full Stack Software Engineer Intern</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
@@ -4700,7 +4672,7 @@
       <c r="E147" s="4" t="inlineStr"/>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>Nov 5</t>
+          <t>Nov 7</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4684,7 @@
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer Intern – AI Engagement Portal</t>
+          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -4735,17 +4707,17 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Valsoft Corporation</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Full Stack Developer Intern – AI Engagement Portal</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -4763,12 +4735,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -4784,24 +4756,24 @@
       <c r="E150" s="4" t="inlineStr"/>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>Nov 4</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Intern - Software Developer</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC, Canada (Remote in Canada)</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -4819,17 +4791,17 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Developer, RBC Amplify 2026</t>
+          <t>Intern - Software Developer</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Montreal, QC, Canada (Remote in Canada)</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
@@ -4840,7 +4812,7 @@
       <c r="E152" s="4" t="inlineStr"/>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>Nov 3</t>
+          <t>Nov 4</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4829,7 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
@@ -4875,17 +4847,17 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Frontend Software Developer Co-op (React.js)</t>
+          <t>Developer, RBC Amplify 2026</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
@@ -4896,7 +4868,7 @@
       <c r="E154" s="4" t="inlineStr"/>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>Oct 30</t>
+          <t>Nov 3</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4880,7 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
+          <t>Frontend Software Developer Co-op (React.js)</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -4941,7 +4913,7 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
@@ -4959,17 +4931,17 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
+          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -4980,19 +4952,19 @@
       <c r="E157" s="4" t="inlineStr"/>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>Oct 29</t>
+          <t>Oct 30</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op, Front End</t>
+          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -5020,7 +4992,7 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Fullstack</t>
+          <t>Software Engineer Co-op, Front End</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -5048,7 +5020,7 @@
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Backend</t>
+          <t>Co-op Software Engineer, Fullstack</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -5071,17 +5043,17 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Summer 2026</t>
+          <t>Co-op Software Engineer, Backend</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
@@ -5092,24 +5064,24 @@
       <c r="E161" s="4" t="inlineStr"/>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>Oct 27</t>
+          <t>Oct 29</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Engineer Internship – Summer 2026</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
@@ -5120,19 +5092,19 @@
       <c r="E162" s="4" t="inlineStr"/>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>Oct 24</t>
+          <t>Oct 27</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -5148,7 +5120,7 @@
       <c r="E163" s="4" t="inlineStr"/>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>Oct 23</t>
+          <t>Oct 24</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5132,7 @@
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
@@ -5176,7 +5148,7 @@
       <c r="E164" s="4" t="inlineStr"/>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>Oct 22</t>
+          <t>Oct 23</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5160,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Cloud Engineer Intern</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -5204,7 +5176,7 @@
       <c r="E165" s="4" t="inlineStr"/>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>Oct 20</t>
+          <t>Oct 22</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5188,7 @@
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>AI Software Developer Intern</t>
+          <t>Cloud Engineer Intern</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -5232,24 +5204,24 @@
       <c r="E166" s="4" t="inlineStr"/>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>Oct 18</t>
+          <t>Oct 20</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>The Athletic</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Engineering Student Intern, Summer 2026</t>
+          <t>AI Software Developer Intern</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
@@ -5260,24 +5232,24 @@
       <c r="E167" s="4" t="inlineStr"/>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>Oct 17</t>
+          <t>Oct 18</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>The Athletic</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>SAP Analytics Cloud Security Engineer Intern</t>
+          <t>Engineering Student Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
@@ -5288,24 +5260,24 @@
       <c r="E168" s="4" t="inlineStr"/>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>Oct 16</t>
+          <t>Oct 17</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Journal Technologies</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Junior Software Developer Co-op</t>
+          <t>SAP Analytics Cloud Security Engineer Intern</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
@@ -5323,17 +5295,17 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>Canada Life</t>
+          <t>Journal Technologies</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Student Position)</t>
+          <t>Junior Software Developer Co-op</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Winnipeg, MB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
@@ -5344,24 +5316,24 @@
       <c r="E170" s="4" t="inlineStr"/>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>Oct 15</t>
+          <t>Oct 16</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Canada Life</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Full-stack Engineering Intern</t>
+          <t>Software Developer (Student Position)</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Winnipeg, MB</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
@@ -5372,7 +5344,7 @@
       <c r="E171" s="4" t="inlineStr"/>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 15</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5356,7 @@
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Backend Engineering Intern</t>
+          <t>Full-stack Engineering Intern</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
@@ -5412,7 +5384,7 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern</t>
+          <t>Backend Engineering Intern</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -5435,17 +5407,17 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern</t>
+          <t>Frontend Engineering Intern</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -5456,19 +5428,19 @@
       <c r="E174" s="4" t="inlineStr"/>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>Oct 10</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Intern – Digital Ship</t>
+          <t>Software Development Intern</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -5484,24 +5456,24 @@
       <c r="E175" s="4" t="inlineStr"/>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>Oct 8</t>
+          <t>Oct 10</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Intern – Digital Ship</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
@@ -5512,24 +5484,24 @@
       <c r="E176" s="4" t="inlineStr"/>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>Oct 7</t>
+          <t>Oct 8</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – Sports Technology</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
@@ -5540,7 +5512,7 @@
       <c r="E177" s="4" t="inlineStr"/>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 7</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5524,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – UFC</t>
+          <t>Software Engineer Intern – Sports Technology</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
@@ -5575,17 +5547,17 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Stateful Systems - Winter 2026</t>
+          <t>Software Engineer Intern – UFC</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
@@ -5596,7 +5568,7 @@
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 6</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5580,7 @@
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Release Engineering - Winter 2026</t>
+          <t>Developer Intern - Stateful Systems - Winter 2026</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
@@ -5636,7 +5608,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement - Winter 2026</t>
+          <t>Developer Intern - Release Engineering - Winter 2026</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -5664,7 +5636,7 @@
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Frameworks - Winter 2026</t>
+          <t>Developer Intern - Platform Advancement - Winter 2026</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
@@ -5692,7 +5664,7 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
+          <t>Developer Intern - Frameworks - Winter 2026</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -5720,7 +5692,7 @@
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - App Launcher - Winter 2026</t>
+          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
@@ -5743,17 +5715,17 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Online Software Engineer Co-op</t>
+          <t>Developer Intern - App Launcher - Winter 2026</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
@@ -5764,24 +5736,24 @@
       <c r="E185" s="4" t="inlineStr"/>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Winter 2026</t>
+          <t>Online Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
@@ -5792,24 +5764,24 @@
       <c r="E186" s="4" t="inlineStr"/>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 4</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
+          <t>Software Development Engineer Internship – Winter 2026</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
@@ -5820,7 +5792,7 @@
       <c r="E187" s="4" t="inlineStr"/>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 3</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5804,7 @@
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – NHL</t>
+          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
@@ -5860,7 +5832,7 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
+          <t>Software Engineer Intern – NHL</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -5883,12 +5855,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Front-end Co-Op</t>
+          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -5904,24 +5876,24 @@
       <c r="E190" s="4" t="inlineStr"/>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>Oct 1</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern – Multiple Teams</t>
+          <t>Software Developer – Front-end Co-Op</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
@@ -5932,24 +5904,24 @@
       <c r="E191" s="4" t="inlineStr"/>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>Sep 23</t>
+          <t>Oct 1</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Datahub)</t>
+          <t>Software Development Intern – Multiple Teams</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
@@ -5960,7 +5932,7 @@
       <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Sep 23</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5944,7 @@
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Quality Assurance)</t>
+          <t>Software Developer Intern (Datahub)</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -6000,7 +5972,7 @@
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Enterprise Applications)</t>
+          <t>Software Developer Intern (Quality Assurance)</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -6023,12 +5995,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern/ Co-op</t>
+          <t>Software Developer Intern (Enterprise Applications)</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -6051,17 +6023,17 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>Hewlett Packard (HP)</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>Associate C++ Software Developer</t>
+          <t>Software Engineering Intern/ Co-op</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
@@ -6072,7 +6044,7 @@
       <c r="E196" s="4" t="inlineStr"/>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>Sep 15</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
@@ -6107,17 +6079,17 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Hewlett Packard (HP)</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>Intern – Software Developer</t>
+          <t>Associate C++ Software Developer</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
@@ -6128,24 +6100,24 @@
       <c r="E198" s="4" t="inlineStr"/>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>Sep 10</t>
+          <t>Sep 15</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Student</t>
+          <t>Intern – Software Developer</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
@@ -6156,24 +6128,24 @@
       <c r="E199" s="4" t="inlineStr"/>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>Sep 08</t>
+          <t>Sep 10</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer Co-op Student</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
@@ -6184,24 +6156,24 @@
       <c r="E200" s="4" t="inlineStr"/>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>Sep 05</t>
+          <t>Sep 08</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer: Internship Opportunities</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
@@ -6212,19 +6184,19 @@
       <c r="E201" s="4" t="inlineStr"/>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>Sep 5</t>
+          <t>Sep 05</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Epic Games</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce Programmer Intern</t>
+          <t>Software Engineer: Internship Opportunities</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
@@ -6240,19 +6212,19 @@
       <c r="E202" s="4" t="inlineStr"/>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>Sep 04</t>
+          <t>Sep 5</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Epic Games</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Ecommerce Programmer Intern</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -6268,24 +6240,24 @@
       <c r="E203" s="4" t="inlineStr"/>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>Sep 01</t>
+          <t>Sep 04</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>TC Energy</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>Computer Science Interns</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
@@ -6296,24 +6268,24 @@
       <c r="E204" s="4" t="inlineStr"/>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 01</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Corpay</t>
+          <t>TC Energy</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Co-op)</t>
+          <t>Computer Science Interns</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -6324,24 +6296,24 @@
       <c r="E205" s="4" t="inlineStr"/>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Aug 31</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Corpay</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer (Co-op)</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
@@ -6352,19 +6324,19 @@
       <c r="E206" s="4" t="inlineStr"/>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>Aug 25</t>
+          <t>Aug 27</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -6380,12 +6352,40 @@
       <c r="E207" s="4" t="inlineStr"/>
       <c r="F207" s="4" t="inlineStr">
         <is>
+          <t>Aug 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Software</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Summer Internship – Various Departments</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>Remote in Canada</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E208" s="4" t="inlineStr"/>
+      <c r="F208" s="4" t="inlineStr">
+        <is>
           <t>Aug 02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F207"/>
+  <autoFilter ref="A1:F208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-05-03
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$211</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F208"/>
+  <dimension ref="A1:F211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stryker</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Systems R&amp;D Engineer Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,24 +535,24 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://stryker.wd1.myworkdayjobs.com/StrykerCareers/job/Burnaby-Canada/Systems-R-D-Engineer-Co-Op_R562620</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677125006</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Apr 17, 2026</t>
+          <t>Apr 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern Fall</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/210894</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677172006</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Apr 17, 2026</t>
+          <t>Apr 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,24 +599,24 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://revvity.wd103.myworkdayjobs.com/External/job/CAD-Remote--ON/Full-Stack-AI-Developer-Intern_JR-043504</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/210840</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Apr 17, 2026</t>
+          <t>Apr 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Test and Manufacturing Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://revvity.wd103.myworkdayjobs.com/External/job/CAD-Remote--ON/Full-Stack-AI-Developer-Intern_JR-044247</t>
+          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Apr 17, 2026</t>
+          <t>Apr 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>OpusClip</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Test and Manufacturing Intern</t>
+          <t>AI Product Manager Intern</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
+          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Apr 16, 2026</t>
+          <t>Apr 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>OpusClip</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager Intern</t>
+          <t>Intern/Co-op - Internal AI Operations</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7808288</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Apr 14, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Intern/Co-op - Internal AI Operations</t>
+          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Ontario, Canada / Remote, Canada</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7808288</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
+          <t>Anthropic Fellows Program, AI Safety</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -771,17 +771,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, AI Safety</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Ontario, Canada / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,29 +791,29 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
+          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Apr 10, 2026</t>
+          <t>Apr 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>BMW Group</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
+          <t>https://www.bmwgroup.jobs/en/jobfinder/job-description-copy.184099.html</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Apr 9, 2026</t>
+          <t>Apr 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BMW Group</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Health Informatics Intern</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,24 +855,24 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmwgroup.jobs/en/jobfinder/job-description-copy.184099.html</t>
+          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apr 7, 2026</t>
+          <t>Mar 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Health Informatics Intern</t>
+          <t>Safety Research Intern</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
+          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mar 10, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Sanctuary AI</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Data Enablement</t>
+          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -919,24 +919,24 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/September-2026---Data-Enablement--CPA----8-month-Co-op---Vancouver_711231WD</t>
+          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Safety Research Intern</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Sanctuary AI</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,140 +983,124 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Tenstorrent</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>IP Product Operations</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Stryker</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Systems R&amp;D Engineer Co-op</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Burnaby, BC</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Apr 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern Fall</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Apr 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Full-Stack AI Developer Intern</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Feb 4, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Apr 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Full-Stack AI Developer Intern</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern, Connected Systems, Summer 2026</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27486?</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Nov 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Rivian</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineering Intern – Applications – Infotainment &amp; Mobile</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.rivian.com/careers-home/jobs/27405</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Nov 5</t>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Apr 17, 2026</t>
         </is>
       </c>
     </row>
@@ -1571,17 +1555,17 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Juniper Square</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer Intern</t>
+          <t>Data Enablement</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1599,17 +1583,17 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>AssetWorks</t>
+          <t>Juniper Square</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>AI Engineer Intern</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1627,17 +1611,17 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>AssetWorks</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1648,24 +1632,24 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Data Engineer</t>
+          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1683,17 +1667,17 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>GIS Intern, Geospatial Services</t>
+          <t>Software Engineering Intern, Data Engineer</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1704,24 +1688,24 @@
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Mar 4, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Developer Co-op</t>
+          <t>GIS Intern, Geospatial Services</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Waterloo, ON / Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1732,24 +1716,24 @@
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Mar 3, 2026</t>
+          <t>Mar 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
+          <t>Developer Co-op</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Waterloo, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1760,7 +1744,7 @@
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Mar 3, 2026</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1756,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack Engineer Intern, Fall 2026</t>
+          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1800,7 +1784,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern, Fall 2026</t>
+          <t>Full-Stack Engineer Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -1823,17 +1807,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>Frontend Engineering Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1844,7 +1828,7 @@
       <c r="E46" s="4" t="inlineStr"/>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1845,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1879,17 +1863,17 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>User Research Co-op</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1900,19 +1884,19 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Feb 26, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Localization Software Developer, Co-Op</t>
+          <t>User Research Co-op</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -1928,24 +1912,24 @@
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Localization Software Developer, Co-Op</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1963,12 +1947,12 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Correlation One</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -1991,17 +1975,17 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Correlation One</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op (Systems)</t>
+          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2012,24 +1996,24 @@
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Feb 24, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
+          <t>Software Engineer Co-op (Systems)</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2040,19 +2024,19 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Feb 19, 2026</t>
+          <t>Feb 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -2075,17 +2059,17 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Critical Mass</t>
+          <t>Jonas Software</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Development Intern</t>
+          <t>Jonas Summer Internship – Various Departments</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2103,17 +2087,17 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Critical Mass</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Automation Development Student</t>
+          <t>Development Intern</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Acheson, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2124,24 +2108,24 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Data Analytics &amp; Automation Development Student</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB / Acheson, AB</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2159,12 +2143,12 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Automation Consulting Intern/Co-op</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -2180,24 +2164,24 @@
       <c r="E58" s="4" t="inlineStr"/>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Feb 17, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>CAE</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>C-MAT-100 Engineering Intern</t>
+          <t>Automation Consulting Intern/Co-op</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Moose Jaw, SK</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2208,24 +2192,24 @@
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Feb 16, 2026</t>
+          <t>Feb 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>CAE</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Application Engineer Test Intern</t>
+          <t>C-MAT-100 Engineering Intern</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Moose Jaw, SK</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2243,17 +2227,17 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>RSM</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Business Intelligence Consulting Associate - Fall 2026</t>
+          <t>Application Engineer Test Intern</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2264,24 +2248,24 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Feb 13, 2026</t>
+          <t>Feb 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>RSM</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Student Digital Systems</t>
+          <t>Business Intelligence Consulting Associate - Fall 2026</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2292,24 +2276,24 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Feb 11, 2026</t>
+          <t>Feb 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Student Digital Systems</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2320,24 +2304,24 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Feb 10, 2026</t>
+          <t>Feb 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Design Methodology Engineering Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2360,7 +2344,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>System Simulation Engineer Intern</t>
+          <t>Design Methodology Engineering Intern</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2383,17 +2367,17 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Fullscript</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>System Simulation Engineer Intern</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Ottawa, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2411,17 +2395,17 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Fullscript</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2432,19 +2416,19 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Feb 9, 2026</t>
+          <t>Feb 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Applied Research Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -2467,17 +2451,17 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Intern, Dto, Enterprise Analytics</t>
+          <t>Applied Research Intern</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2500,7 +2484,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
+          <t>Intern, Dto, Enterprise Analytics</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -2528,7 +2512,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Intern, Data &amp; Integrations</t>
+          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -2551,12 +2535,12 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Design Validation Intern/Co-op</t>
+          <t>Intern, Data &amp; Integrations</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -2579,17 +2563,17 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Mikata Health</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Data Science Intern</t>
+          <t>Design Validation Intern/Co-op</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2607,17 +2591,17 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Instacart</t>
+          <t>Mikata Health</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Data Science PhD Intern</t>
+          <t>Healthcare Data Science Intern</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2628,19 +2612,19 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Feb 5, 2026</t>
+          <t>Feb 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Instacart</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Client Secrets Management</t>
+          <t>Data Science PhD Intern</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -2656,24 +2640,24 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Feb 3, 2026</t>
+          <t>Feb 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Developer Intern - Client Secrets Management</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2684,24 +2668,24 @@
       <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Feb 2, 2026</t>
+          <t>Feb 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Data Intern - Enterprise Analytics</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2719,17 +2703,17 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Veralto</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Co-Op Intern</t>
+          <t>Data Intern - Enterprise Analytics</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2740,24 +2724,24 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Feb 1, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Veralto</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Knox</t>
+          <t>Machine Learning Co-Op Intern</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2768,7 +2752,7 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Jan 30, 2026</t>
+          <t>Feb 1, 2026</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2764,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Trust Platforms</t>
+          <t>Developer Intern - Knox</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -2808,7 +2792,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Extension Excellence</t>
+          <t>Developer Intern - Trust Platforms</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -2836,7 +2820,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Insights</t>
+          <t>Developer Intern - Extension Excellence</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -2864,7 +2848,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement</t>
+          <t>Developer Intern - Insights</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -2892,7 +2876,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Device Security</t>
+          <t>Developer Intern - Platform Advancement</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -2920,7 +2904,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Billing &amp; Payments</t>
+          <t>Developer Intern - Device Security</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2948,7 +2932,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Data &amp; Access</t>
+          <t>Developer Intern - Billing &amp; Payments</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -2971,17 +2955,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Student Engineer</t>
+          <t>Developer Intern - Data &amp; Access</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2999,17 +2983,17 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Voldex</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Game Developer Intern</t>
+          <t>Student Engineer</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3020,19 +3004,19 @@
       <c r="E88" s="4" t="inlineStr"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Jan 29, 2026</t>
+          <t>Jan 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>GE Healthcare</t>
+          <t>Voldex</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Field Service Apprentice</t>
+          <t>Game Developer Intern</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -3048,24 +3032,24 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Jan 28, 2026</t>
+          <t>Jan 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>GE Healthcare</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-Op</t>
+          <t>Field Service Apprentice</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3083,17 +3067,17 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern/Co-op</t>
+          <t>Software Engineer Co-Op</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3104,24 +3088,24 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Jan 26, 2026</t>
+          <t>Jan 28, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>BC Pensions</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Application Developer Intern/Co-op</t>
+          <t>Software Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -3139,17 +3123,17 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>BC Pensions</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Support Enablement Engineer Intern</t>
+          <t>Application Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3160,19 +3144,19 @@
       <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Jan 23, 2026</t>
+          <t>Jan 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Intern Full Stack Developer</t>
+          <t>Support Enablement Engineer Intern</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -3195,12 +3179,12 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Allstate Insurance Company</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Data Governance Intern/Co-op</t>
+          <t>Intern Full Stack Developer</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -3216,7 +3200,7 @@
       <c r="E95" s="4" t="inlineStr"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Jan 22, 2026</t>
+          <t>Jan 23, 2026</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3212,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Provincial Product Analyst Co-op</t>
+          <t>Data Governance Intern/Co-op</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -3251,17 +3235,17 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Allstate Insurance Company</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern - Summer 2026</t>
+          <t>Provincial Product Analyst Co-op</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3272,7 +3256,7 @@
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Jan 21, 2026</t>
+          <t>Jan 22, 2026</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3268,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern - Summer 2026</t>
+          <t>Production Engineering Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -3312,7 +3296,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Graduate Production Engineer Research Intern</t>
+          <t>Studio Talent Group Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -3340,7 +3324,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Technical Assistant Intern - Summer 2026</t>
+          <t>Graduate Production Engineer Research Intern</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -3363,17 +3347,17 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>BMO</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Co-op/Internship</t>
+          <t>Technical Assistant Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3384,19 +3368,19 @@
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Jan 19, 2026</t>
+          <t>Jan 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>BMO</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Developer – Co-op/Internship</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -3419,17 +3403,17 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Engineering Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3440,24 +3424,24 @@
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Jan 17, 2026</t>
+          <t>Jan 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>The Boeing Company</t>
+          <t>Boomi</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Engineering Intern</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -3468,7 +3452,7 @@
       <c r="E104" s="4" t="inlineStr"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Jan 16, 2026</t>
+          <t>Jan 17, 2026</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3464,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Data Engineering Intern</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -3508,7 +3492,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Data Science Business Operations Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -3531,17 +3515,17 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>The Boeing Company</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Systems Analyst</t>
+          <t>Data Science Business Operations Intern</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -3559,12 +3543,12 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>AI/ML Coop/Intern</t>
+          <t>Systems Analyst</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -3587,17 +3571,17 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Enbridge</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>SharePoint &amp; Document Management Support - Summer Student</t>
+          <t>AI/ML Coop/Intern</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -3615,17 +3599,17 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Enbridge</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Game Creation SW Engineer Intern</t>
+          <t>SharePoint &amp; Document Management Support - Summer Student</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -3636,24 +3620,24 @@
       <c r="E110" s="4" t="inlineStr"/>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>Jan 15, 2026</t>
+          <t>Jan 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
+          <t>Game Creation SW Engineer Intern</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -3676,7 +3660,7 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -3699,17 +3683,17 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -3720,19 +3704,19 @@
       <c r="E113" s="4" t="inlineStr"/>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>Jan 13</t>
+          <t>Jan 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer - Internship Opportunities</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
@@ -3748,24 +3732,24 @@
       <c r="E114" s="4" t="inlineStr"/>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Jan 12</t>
+          <t>Jan 13</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineering Intern</t>
+          <t>Software Engineer - Internship Opportunities</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -3776,24 +3760,24 @@
       <c r="E115" s="4" t="inlineStr"/>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Jan 9</t>
+          <t>Jan 12</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Triton Compiler Engineering Intern</t>
+          <t>Systems Software Engineering Intern</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Remote in Canada</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3811,17 +3795,17 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - Co-op - Full Stack</t>
+          <t>Triton Compiler Engineering Intern</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3844,7 +3828,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
+          <t>Software Developer - Co-op - Full Stack</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -3872,7 +3856,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - C++ - Co-op</t>
+          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -3895,12 +3879,12 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer - C++ - Co-op</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
@@ -3923,17 +3907,17 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op/Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -3944,24 +3928,24 @@
       <c r="E121" s="4" t="inlineStr"/>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>Jan 8</t>
+          <t>Jan 9</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -3979,7 +3963,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -4000,14 +3984,14 @@
       <c r="E123" s="4" t="inlineStr"/>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>Jan 7</t>
+          <t>Jan 8</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -4028,24 +4012,24 @@
       <c r="E124" s="4" t="inlineStr"/>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>Jan 6</t>
+          <t>Jan 7</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern/Co-op - Oracle APEX</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -4056,24 +4040,24 @@
       <c r="E125" s="4" t="inlineStr"/>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>Jan 5</t>
+          <t>Jan 6</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Intern/Co-op - Oracle APEX</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
@@ -4091,17 +4075,17 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>BDC</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -4119,17 +4103,17 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>BDC</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
+          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -4140,7 +4124,7 @@
       <c r="E128" s="4" t="inlineStr"/>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>Dec 20</t>
+          <t>Jan 5</t>
         </is>
       </c>
     </row>
@@ -4152,12 +4136,12 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
+          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -4175,17 +4159,17 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Accenture</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern - Echo</t>
+          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -4196,24 +4180,24 @@
       <c r="E130" s="4" t="inlineStr"/>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>Dec 18</t>
+          <t>Dec 20</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer Intern - Echo</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -4224,24 +4208,24 @@
       <c r="E131" s="4" t="inlineStr"/>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>Dec 17</t>
+          <t>Dec 18</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - AI/ML QVS</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -4252,24 +4236,24 @@
       <c r="E132" s="4" t="inlineStr"/>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>Dec 15</t>
+          <t>Dec 17</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>RBC Borealis - Machine Learning Software Engineer</t>
+          <t>Software Engineer Intern - AI/ML QVS</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -4280,24 +4264,24 @@
       <c r="E133" s="4" t="inlineStr"/>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>Dec 12</t>
+          <t>Dec 15</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Applications - Summer 2026</t>
+          <t>RBC Borealis - Machine Learning Software Engineer</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -4320,7 +4304,7 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
+          <t>Software Engineering Intern, Applications - Summer 2026</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
@@ -4343,12 +4327,12 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern</t>
+          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
@@ -4376,7 +4360,7 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern</t>
+          <t>Production Engineering Intern</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -4392,19 +4376,19 @@
       <c r="E137" s="4" t="inlineStr"/>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>Dec 11</t>
+          <t>Dec 12</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>DataVisor</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Backend Software Engineer Internship</t>
+          <t>Studio Talent Group Intern</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
@@ -4420,24 +4404,24 @@
       <c r="E138" s="4" t="inlineStr"/>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>Dec 10</t>
+          <t>Dec 11</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>DataVisor</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op</t>
+          <t>Backend Software Engineer Internship</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Kitchener, ON / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
@@ -4455,17 +4439,17 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern - Summer 2026</t>
+          <t>Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Ottawa, ON / Calgary, AB / Vancouver, BC / Victoria, BC</t>
+          <t>Kitchener, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -4476,24 +4460,24 @@
       <c r="E140" s="4" t="inlineStr"/>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>Dec 9</t>
+          <t>Dec 10</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Computer Engineering Intern - TFE Service Team</t>
+          <t>Software Development Engineer Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Toronto, ON / Ottawa, ON / Calgary, AB / Vancouver, BC / Victoria, BC</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -4504,24 +4488,24 @@
       <c r="E141" s="4" t="inlineStr"/>
       <c r="F141" s="4" t="inlineStr">
         <is>
-          <t>Dec 1</t>
+          <t>Dec 9</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>Ticketmaster</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Computer Engineering Intern - TFE Service Team</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
@@ -4532,24 +4516,24 @@
       <c r="E142" s="4" t="inlineStr"/>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>Nov 26</t>
+          <t>Dec 1</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Ticketmaster</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineer Intern/Co-op</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
@@ -4560,24 +4544,24 @@
       <c r="E143" s="4" t="inlineStr"/>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>Nov 15</t>
+          <t>Nov 26</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>Volaris Group</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Systems Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Mississauga, ON, Canada / Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
@@ -4588,24 +4572,24 @@
       <c r="E144" s="4" t="inlineStr"/>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>Nov 14</t>
+          <t>Nov 15</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Volaris Group</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Co-Op/Intern – Software Development – Winter 2026</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Calgary, AB / Vancouver, BC</t>
+          <t>Mississauga, ON, Canada / Remote in Canada</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
@@ -4616,24 +4600,24 @@
       <c r="E145" s="4" t="inlineStr"/>
       <c r="F145" s="4" t="inlineStr">
         <is>
-          <t>Nov 13</t>
+          <t>Nov 14</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Software Automation Engineering Intern, Summer 2026</t>
+          <t>Co-Op/Intern – Software Development – Winter 2026</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Calgary, AB / Vancouver, BC</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
@@ -4651,12 +4635,12 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>Transcarent</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Software Engineer Intern</t>
+          <t>Software Engineering Intern, Connected Systems, Summer 2026</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -4672,24 +4656,24 @@
       <c r="E147" s="4" t="inlineStr"/>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>Nov 7</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Valsoft Corporation</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
+          <t>Software Automation Engineering Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
@@ -4700,24 +4684,24 @@
       <c r="E148" s="4" t="inlineStr"/>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>Nov 5</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>Valsoft Corporation</t>
+          <t>Transcarent</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer Intern – AI Engagement Portal</t>
+          <t>Full Stack Software Engineer Intern</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -4728,24 +4712,24 @@
       <c r="E149" s="4" t="inlineStr"/>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>Nov 5</t>
+          <t>Nov 7</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Valsoft Corporation</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -4763,17 +4747,17 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Valsoft Corporation</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Full Stack Developer Intern – AI Engagement Portal</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -4784,24 +4768,24 @@
       <c r="E151" s="4" t="inlineStr"/>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>Nov 4</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Intern - Software Developer</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC, Canada (Remote in Canada)</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
@@ -4812,19 +4796,19 @@
       <c r="E152" s="4" t="inlineStr"/>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>Nov 4</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Developer, RBC Amplify 2026</t>
+          <t>Software Engineering Intern, Applications, Infotainment &amp; Mobile</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -4840,24 +4824,24 @@
       <c r="E153" s="4" t="inlineStr"/>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>Nov 3</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Developer, RBC Amplify 2026</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
@@ -4868,24 +4852,24 @@
       <c r="E154" s="4" t="inlineStr"/>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>Nov 3</t>
+          <t>Nov 4</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Frontend Software Developer Co-op (React.js)</t>
+          <t>Intern - Software Developer</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Montreal, QC, Canada (Remote in Canada)</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
@@ -4896,19 +4880,19 @@
       <c r="E155" s="4" t="inlineStr"/>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>Oct 30</t>
+          <t>Nov 4</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
+          <t>Developer, RBC Amplify 2026</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -4924,24 +4908,24 @@
       <c r="E156" s="4" t="inlineStr"/>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>Oct 30</t>
+          <t>Nov 3</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
+          <t>Developer, RBC Amplify 2026</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -4952,19 +4936,19 @@
       <c r="E157" s="4" t="inlineStr"/>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>Oct 30</t>
+          <t>Nov 3</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
+          <t>Frontend Software Developer Co-op (React.js)</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -4980,19 +4964,19 @@
       <c r="E158" s="4" t="inlineStr"/>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>Oct 29</t>
+          <t>Oct 30</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op, Front End</t>
+          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -5008,24 +4992,24 @@
       <c r="E159" s="4" t="inlineStr"/>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>Oct 29</t>
+          <t>Oct 30</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Fullstack</t>
+          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
@@ -5036,19 +5020,19 @@
       <c r="E160" s="4" t="inlineStr"/>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>Oct 29</t>
+          <t>Oct 30</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Backend</t>
+          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
@@ -5071,17 +5055,17 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Summer 2026</t>
+          <t>Software Engineer Co-op, Front End</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
@@ -5092,19 +5076,19 @@
       <c r="E162" s="4" t="inlineStr"/>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>Oct 27</t>
+          <t>Oct 29</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Co-op Software Engineer, Fullstack</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -5120,19 +5104,19 @@
       <c r="E163" s="4" t="inlineStr"/>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>Oct 24</t>
+          <t>Oct 29</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
+          <t>Co-op Software Engineer, Backend</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
@@ -5148,24 +5132,24 @@
       <c r="E164" s="4" t="inlineStr"/>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>Oct 23</t>
+          <t>Oct 29</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Software Development Engineer Internship – Summer 2026</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
@@ -5176,19 +5160,19 @@
       <c r="E165" s="4" t="inlineStr"/>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>Oct 22</t>
+          <t>Oct 27</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Cloud Engineer Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -5204,7 +5188,7 @@
       <c r="E166" s="4" t="inlineStr"/>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>Oct 20</t>
+          <t>Oct 24</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5200,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>AI Software Developer Intern</t>
+          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -5232,24 +5216,24 @@
       <c r="E167" s="4" t="inlineStr"/>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>Oct 18</t>
+          <t>Oct 23</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>The Athletic</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Engineering Student Intern, Summer 2026</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
@@ -5260,7 +5244,7 @@
       <c r="E168" s="4" t="inlineStr"/>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>Oct 17</t>
+          <t>Oct 22</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5256,7 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>SAP Analytics Cloud Security Engineer Intern</t>
+          <t>Cloud Engineer Intern</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -5288,24 +5272,24 @@
       <c r="E169" s="4" t="inlineStr"/>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>Oct 16</t>
+          <t>Oct 20</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>Journal Technologies</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Junior Software Developer Co-op</t>
+          <t>AI Software Developer Intern</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
@@ -5316,24 +5300,24 @@
       <c r="E170" s="4" t="inlineStr"/>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>Oct 16</t>
+          <t>Oct 18</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Canada Life</t>
+          <t>The Athletic</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Student Position)</t>
+          <t>Engineering Student Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Winnipeg, MB</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
@@ -5344,24 +5328,24 @@
       <c r="E171" s="4" t="inlineStr"/>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>Oct 15</t>
+          <t>Oct 17</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Full-stack Engineering Intern</t>
+          <t>SAP Analytics Cloud Security Engineer Intern</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
@@ -5372,24 +5356,24 @@
       <c r="E172" s="4" t="inlineStr"/>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 16</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Journal Technologies</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Backend Engineering Intern</t>
+          <t>Junior Software Developer Co-op</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
@@ -5400,24 +5384,24 @@
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 16</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Canada Life</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern</t>
+          <t>Software Developer (Student Position)</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Winnipeg, MB</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -5428,24 +5412,24 @@
       <c r="E174" s="4" t="inlineStr"/>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 15</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern</t>
+          <t>Full-stack Engineering Intern</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
@@ -5456,24 +5440,24 @@
       <c r="E175" s="4" t="inlineStr"/>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>Oct 10</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Intern – Digital Ship</t>
+          <t>Backend Engineering Intern</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
@@ -5484,19 +5468,19 @@
       <c r="E176" s="4" t="inlineStr"/>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>Oct 8</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Frontend Engineering Intern</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -5512,7 +5496,7 @@
       <c r="E177" s="4" t="inlineStr"/>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>Oct 7</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5508,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – Sports Technology</t>
+          <t>Software Development Intern</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
@@ -5540,19 +5524,19 @@
       <c r="E178" s="4" t="inlineStr"/>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 10</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – UFC</t>
+          <t>Intern – Digital Ship</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -5568,19 +5552,19 @@
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 8</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Stateful Systems - Winter 2026</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
@@ -5596,24 +5580,24 @@
       <c r="E180" s="4" t="inlineStr"/>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 7</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Release Engineering - Winter 2026</t>
+          <t>Software Engineer Intern – Sports Technology</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
@@ -5624,24 +5608,24 @@
       <c r="E181" s="4" t="inlineStr"/>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 6</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement - Winter 2026</t>
+          <t>Software Engineer Intern – UFC</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
@@ -5652,7 +5636,7 @@
       <c r="E182" s="4" t="inlineStr"/>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 6</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5648,7 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Frameworks - Winter 2026</t>
+          <t>Developer Intern - Stateful Systems - Winter 2026</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -5692,7 +5676,7 @@
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
+          <t>Developer Intern - Release Engineering - Winter 2026</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
@@ -5720,7 +5704,7 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - App Launcher - Winter 2026</t>
+          <t>Developer Intern - Platform Advancement - Winter 2026</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
@@ -5743,17 +5727,17 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Online Software Engineer Co-op</t>
+          <t>Developer Intern - Frameworks - Winter 2026</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
@@ -5764,24 +5748,24 @@
       <c r="E186" s="4" t="inlineStr"/>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Winter 2026</t>
+          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
@@ -5792,24 +5776,24 @@
       <c r="E187" s="4" t="inlineStr"/>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
+          <t>Developer Intern - App Launcher - Winter 2026</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
@@ -5820,7 +5804,7 @@
       <c r="E188" s="4" t="inlineStr"/>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5816,7 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – NHL</t>
+          <t>Online Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -5848,24 +5832,24 @@
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 4</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
+          <t>Software Development Engineer Internship – Winter 2026</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
@@ -5876,19 +5860,19 @@
       <c r="E190" s="4" t="inlineStr"/>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 3</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Front-end Co-Op</t>
+          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -5904,24 +5888,24 @@
       <c r="E191" s="4" t="inlineStr"/>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>Oct 1</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern – Multiple Teams</t>
+          <t>Software Engineer Intern – NHL</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
@@ -5932,24 +5916,24 @@
       <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>Sep 23</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Datahub)</t>
+          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
@@ -5960,24 +5944,24 @@
       <c r="E193" s="4" t="inlineStr"/>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Quality Assurance)</t>
+          <t>Software Developer – Front-end Co-Op</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
@@ -5988,24 +5972,24 @@
       <c r="E194" s="4" t="inlineStr"/>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Oct 1</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Enterprise Applications)</t>
+          <t>Software Development Intern – Multiple Teams</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
@@ -6016,19 +6000,19 @@
       <c r="E195" s="4" t="inlineStr"/>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Sep 23</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern/ Co-op</t>
+          <t>Software Developer Intern (Datahub)</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -6051,17 +6035,17 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Hewlett Packard (HP)</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>Associate C++ Software Developer</t>
+          <t>Software Developer Intern (Quality Assurance)</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
@@ -6072,24 +6056,24 @@
       <c r="E197" s="4" t="inlineStr"/>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>Sep 15</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Hewlett Packard (HP)</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>Associate C++ Software Developer</t>
+          <t>Software Developer Intern (Enterprise Applications)</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
@@ -6100,24 +6084,24 @@
       <c r="E198" s="4" t="inlineStr"/>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>Sep 15</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>Intern – Software Developer</t>
+          <t>Software Engineering Intern/ Co-op</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
@@ -6128,19 +6112,19 @@
       <c r="E199" s="4" t="inlineStr"/>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>Sep 10</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Hewlett Packard (HP)</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Student</t>
+          <t>Associate C++ Software Developer</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -6156,24 +6140,24 @@
       <c r="E200" s="4" t="inlineStr"/>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>Sep 08</t>
+          <t>Sep 15</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Hewlett Packard (HP)</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Associate C++ Software Developer</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
@@ -6184,24 +6168,24 @@
       <c r="E201" s="4" t="inlineStr"/>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>Sep 05</t>
+          <t>Sep 15</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer: Internship Opportunities</t>
+          <t>Intern – Software Developer</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
@@ -6212,19 +6196,19 @@
       <c r="E202" s="4" t="inlineStr"/>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>Sep 5</t>
+          <t>Sep 10</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Epic Games</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce Programmer Intern</t>
+          <t>Software Engineer Co-op Student</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -6240,24 +6224,24 @@
       <c r="E203" s="4" t="inlineStr"/>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>Sep 04</t>
+          <t>Sep 08</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
@@ -6268,24 +6252,24 @@
       <c r="E204" s="4" t="inlineStr"/>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>Sep 01</t>
+          <t>Sep 05</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>TC Energy</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>Computer Science Interns</t>
+          <t>Software Engineer: Internship Opportunities</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -6296,19 +6280,19 @@
       <c r="E205" s="4" t="inlineStr"/>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 5</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>Corpay</t>
+          <t>Epic Games</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Co-op)</t>
+          <t>Ecommerce Programmer Intern</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
@@ -6324,14 +6308,14 @@
       <c r="E206" s="4" t="inlineStr"/>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Sep 04</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
@@ -6341,7 +6325,7 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
@@ -6352,24 +6336,24 @@
       <c r="E207" s="4" t="inlineStr"/>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>Aug 25</t>
+          <t>Sep 01</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>TC Energy</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Computer Science Interns</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
@@ -6380,12 +6364,96 @@
       <c r="E208" s="4" t="inlineStr"/>
       <c r="F208" s="4" t="inlineStr">
         <is>
+          <t>Aug 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>Corpay</t>
+        </is>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>Software Developer (Co-op)</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E209" s="4" t="inlineStr"/>
+      <c r="F209" s="4" t="inlineStr">
+        <is>
+          <t>Aug 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>Dropbox</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>Remote in Canada</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E210" s="4" t="inlineStr"/>
+      <c r="F210" s="4" t="inlineStr">
+        <is>
+          <t>Aug 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Software</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Summer Internship – Various Departments</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>Remote in Canada</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E211" s="4" t="inlineStr"/>
+      <c r="F211" s="4" t="inlineStr">
+        <is>
           <t>Aug 02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F208"/>
+  <autoFilter ref="A1:F211"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-05-31
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>NAV CANADA</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Software Engineer Co-op</t>
+          <t>Technical Services Technologist Trainee</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://rbc.wd3.myworkdayjobs.com/ExternalPrivatePostingStudents/job/TORONTO-Ontario-Canada/XMLNAME-2026-Fall-Student-Opportunities-RBC-Borealis---Machine-Learning-Software-Engineer--4-8-Months_R-0000168679</t>
+          <t>https://navcanada.wd10.myworkdayjobs.com/NAV_Careers/job/Calgary/Technical-Services-Technologist-Trainee_JR-8110</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>May 23, 2026</t>
+          <t>May 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NAV CANADA</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Technical Services Technologist Trainee</t>
+          <t>Systems Engineer Co-op</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://navcanada.wd10.myworkdayjobs.com/NAV_Careers/job/Calgary/Technical-Services-Technologist-Trainee_JR-8110</t>
+          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Systems-Engineer--Co-Op_R65120-1</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>May 21, 2026</t>
+          <t>May 20, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Systems Engineer Co-op</t>
+          <t>Engineering/Development Intern/Co-op</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Systems-Engineer--Co-Op_R65120-1</t>
+          <t>https://mksinst.wd1.myworkdayjobs.com/MKSCareersUniversity/job/Canada-Richmond/XMLNAME-2026-Fall-Engineering-Development-Intern-Co-op_R14406</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -611,17 +611,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Engineering/Development Intern/Co-op</t>
+          <t>Software Development Co-op, Firmware Development and Test</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,12 +631,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://mksinst.wd1.myworkdayjobs.com/MKSCareersUniversity/job/Canada-Richmond/XMLNAME-2026-Fall-Engineering-Development-Intern-Co-op_R14406</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000127255469</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>May 20, 2026</t>
+          <t>May 19, 2026</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Software Development Co-op, Firmware Development and Test</t>
+          <t>Software Development and Test Co-op</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000127255469</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000127255509</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -675,17 +675,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Software Development and Test Co-op</t>
+          <t>Data &amp; Analytics Co-op/Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Montreal, QC / Calgary, AB / Toronto, ON / Vancouver, BC / Ottawa, ON / Oakville, ON / Halifax, NS</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000127255509</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--September-2026-_JR6295</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>May 19, 2026</t>
+          <t>May 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BDO Canada</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Co-op/Intern</t>
+          <t>Data Analytics Co-op</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Montreal, QC / Calgary, AB / Toronto, ON / Vancouver, BC / Ottawa, ON / Oakville, ON / Halifax, NS</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--September-2026-_JR6295</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20111</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Co-op</t>
+          <t>IT Analytics Co-op</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20111</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20112</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -771,17 +771,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>IT Analytics Co-op</t>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20112</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Risk-Analytics-Solutions-Co-op-Internship--Fall-2026---Winter-2027-_JR101491</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Risk-Analytics-Solutions-Co-op-Internship--Fall-2026---Winter-2027-_JR101491</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Risk-Reporting---Data-Co-op-Internship--Fall-2026---Winter-2027-_JR101493</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Enterprise Solutions Software Engineer Co-op/Internship</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Victoria, BC / Vancouver, BC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Risk-Reporting---Data-Co-op-Internship--Fall-2026---Winter-2027-_JR101493</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Enterprise-Solutions--Software-Engineer-Co-op-Internship--Fall-2026-_JR101472</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Solutions Software Engineer Co-op/Internship</t>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Enterprise-Solutions--Software-Engineer-Co-op-Internship--Fall-2026-_JR101472</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Data---Analytics-Engineer-Co-op--Internship--Fall-2026-and-or-Winter-2027-_JR101481</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -899,17 +899,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Machine Learning Intern/Co-op</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Data---Analytics-Engineer-Co-op--Internship--Fall-2026-and-or-Winter-2027-_JR101481</t>
+          <t>https://jobs.ashbyhq.com/cohere/36d1f52f-8270-4652-adf5-5303a0ff341b/application</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>May 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Intern/Co-op</t>
+          <t>Design Technologist Co-op</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/36d1f52f-8270-4652-adf5-5303a0ff341b/application</t>
+          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Design-Technologist---2026-Coop_R64943</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -963,17 +963,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Design Technologist Co-op</t>
+          <t>Software Development Engineer Co-op</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,24 +983,24 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Design-Technologist---2026-Coop_R64943</t>
+          <t>https://job-boards.greenhouse.io/athinkingape/jobs/7918788</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>May 13, 2026</t>
+          <t>May 12, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Co-op</t>
+          <t>Payments Engineer Intern</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/athinkingape/jobs/7918788</t>
+          <t>https://jobs.ashbyhq.com/super.com/6a0dc25b-6eb2-411e-a862-6b083d9bad3c/</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>May 12, 2026</t>
+          <t>May 11, 2026</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Payments Engineer Intern</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/6a0dc25b-6eb2-411e-a862-6b083d9bad3c/</t>
+          <t>https://jobs.ashbyhq.com/super.com/5060f2c1-a0ca-44a9-90b6-647ead38d2e8/</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Software Engineer Intern, Data</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/5060f2c1-a0ca-44a9-90b6-647ead38d2e8/</t>
+          <t>https://jobs.ashbyhq.com/super.com/026d7e42-85b6-4baa-bab8-bf3f6d10bc0d/</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Data</t>
+          <t>Quality Intern, Travel &amp; AI Enablement</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/026d7e42-85b6-4baa-bab8-bf3f6d10bc0d/</t>
+          <t>https://jobs.ashbyhq.com/super.com/3854181c-a5d4-440f-9252-499749acf7c9/</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Quality Intern, Travel &amp; AI Enablement</t>
+          <t>Software Engineer Intern, Product, Full-Stack</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/3854181c-a5d4-440f-9252-499749acf7c9/</t>
+          <t>https://jobs.ashbyhq.com/super.com/8179b5ad-9074-4d96-aa92-366cf12ab5d5/</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Product, Full-Stack</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/8179b5ad-9074-4d96-aa92-366cf12ab5d5/</t>
+          <t>https://jobs.ashbyhq.com/super.com/1fdfd963-c5cb-49a0-be9a-76826aabf922/</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Data Analytics Intern, Risk &amp; Fraud</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/1fdfd963-c5cb-49a0-be9a-76826aabf922/</t>
+          <t>https://jobs.ashbyhq.com/super.com/8355a2fc-34bc-45b0-b8d6-39e558940cef/</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern, Risk &amp; Fraud</t>
+          <t>Systems Integration Engineer Co-op</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1239,29 +1239,29 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/8355a2fc-34bc-45b0-b8d6-39e558940cef/</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000125181520</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>May 11, 2026</t>
+          <t>May 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Occidental Petroleum</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Systems Integration Engineer Co-op</t>
+          <t>Process Systems Engineering Co-op, Automation &amp; Data Integration</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Squamish, BC</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1271,29 +1271,29 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000125181520</t>
+          <t>https://oxy.wd5.myworkdayjobs.com/Corporate/job/Squamish/Process-Systems-Engineering--Automation---Data-Integration---Co-op_JR108371</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>May 7, 2026</t>
+          <t>May 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Occidental Petroleum</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Process Systems Engineering Co-op, Automation &amp; Data Integration</t>
+          <t>Software Engineering Developer Co-op</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Squamish, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://oxy.wd5.myworkdayjobs.com/Corporate/job/Squamish/Process-Systems-Engineering--Automation---Data-Integration---Co-op_JR108371</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000124931443</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1315,17 +1315,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Developer Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000124931443</t>
+          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-Op_R-28476</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>May 6, 2026</t>
+          <t>May 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Design Methodology Engineer Intern</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-Op_R-28476</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Methodology-Engineering-Intern_JR0283526</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Design Methodology Engineer Intern</t>
+          <t>Firmware Development Engineer Intern</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Methodology-Engineering-Intern_JR0283526</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Engineer_JR0283529</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Firmware Development Engineer Intern</t>
+          <t>Design Emulation Engineer Intern</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Engineer_JR0283529</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Emulation-Engineer_JR0283530</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1443,17 +1443,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Diligent Corporation</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Design Emulation Engineer Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Emulation-Engineer_JR0283530</t>
+          <t>https://job-boards.greenhouse.io/diligentcorporation/jobs/5987823004</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1475,17 +1475,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Diligent Corporation</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Design Verification Engineer Intern</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1495,29 +1495,29 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/diligentcorporation/jobs/5987823004</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Verification-Engineering-Intern_JR0283524</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>May 5, 2026</t>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Design Verification Engineer Intern</t>
+          <t>Data Scientist Intern/Co-op</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Verification-Engineering-Intern_JR0283524</t>
+          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/Data-Scientist-I--4-Month-Co-op-Internship--Fall-2026-_R152902-1</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1539,12 +1539,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist Intern/Co-op</t>
+          <t>Application Engineer Co-op</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/Data-Scientist-I--4-Month-Co-op-Internship--Fall-2026-_R152902-1</t>
+          <t>https://jobs.lever.co/arcteryx.com/d8c59871-eabf-4505-aa6f-9ca34aa9154c/</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1571,17 +1571,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Application Engineer Co-op</t>
+          <t>Data Analyst Intern, Customer Success Operations</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/arcteryx.com/d8c59871-eabf-4505-aa6f-9ca34aa9154c/</t>
+          <t>https://job-boards.greenhouse.io/internshiplist2000/jobs/5185496008</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1603,17 +1603,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst Intern, Customer Success Operations</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1623,12 +1623,12 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/internshiplist2000/jobs/5185496008</t>
+          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>May 1, 2026</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Research Internship</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
+          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1667,17 +1667,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Research Internship</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677125006</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>May 1, 2026</t>
+          <t>Apr 29, 2026</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677125006</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677172006</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1731,12 +1731,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4677172006</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/210840</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Apr 29, 2026</t>
+          <t>Apr 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Test and Manufacturing Intern</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,29 +1783,29 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/210840</t>
+          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Apr 24, 2026</t>
+          <t>Apr 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>OpusClip</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Test and Manufacturing Intern</t>
+          <t>AI Product Manager Intern</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1815,24 +1815,24 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://calix.wd1.myworkdayjobs.com/External/job/Remote---USA/Test-and-Manufacturing-Intern_R-11632</t>
+          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Apr 16, 2026</t>
+          <t>Apr 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>OpusClip</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager Intern</t>
+          <t>Intern/Co-op - Internal AI Operations</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1847,29 +1847,29 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/opusclip/5875cb24-d27e-4f79-bc2d-a664f5f02298/</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7808288</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Apr 14, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Intern/Co-op - Internal AI Operations</t>
+          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Ontario, Canada / Remote, Canada</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7808288</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
+          <t>Anthropic Fellows Program, AI Safety</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1923,17 +1923,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, AI Safety</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Ontario, Canada / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1943,29 +1943,29 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
+          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Apr 10, 2026</t>
+          <t>Apr 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>BMW Group</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1975,29 +1975,29 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
+          <t>https://www.bmwgroup.jobs/en/jobfinder/job-description-copy.184099.html</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Apr 9, 2026</t>
+          <t>Apr 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BMW Group</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Health Informatics Intern</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2007,24 +2007,24 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmwgroup.jobs/en/jobfinder/job-description-copy.184099.html</t>
+          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Apr 7, 2026</t>
+          <t>Mar 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Health Informatics Intern</t>
+          <t>Safety Research Intern</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2039,29 +2039,29 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://harriscomputer.wd3.myworkdayjobs.com/1/job/Remote---Saskatchewan/Intern_R0040214</t>
+          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Mar 10, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Sanctuary AI</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Safety Research Intern</t>
+          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2071,29 +2071,29 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/f172c484-071a-4a90-a138-e064d69608ba/</t>
+          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Sanctuary AI</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2103,24 +2103,24 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/sanctuary/0e60fef6-a3e1-4a81-8345-75cd120e5b40</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Tenstorrent</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>IP Product Operations</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2135,44 +2135,40 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Feb 4, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>RBC</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Machine Learning Software Engineer Co-op</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>May 23, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-07-05
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -2659,7 +2659,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Diligent Corporation</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2679,24 +2679,24 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/diligentcorporation/jobs/5987823004</t>
+          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>May 5, 2026</t>
+          <t>May 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Design Verification Engineer Intern</t>
+          <t>Research Internship</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2711,29 +2711,29 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Design-Verification-Engineering-Intern_JR0283524</t>
+          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>May 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist Intern/Co-op</t>
+          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Ontario, Canada / Remote, Canada</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2743,29 +2743,29 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/Data-Scientist-I--4-Month-Co-op-Internship--Fall-2026-_R152902-1</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Application Engineer Co-op</t>
+          <t>Anthropic Fellows Program, AI Safety</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Ontario, Canada / Remote, Canada</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2775,29 +2775,29 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/arcteryx.com/d8c59871-eabf-4505-aa6f-9ca34aa9154c/</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst Intern, Customer Success Operations</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2807,24 +2807,24 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/internshiplist2000/jobs/5185496008</t>
+          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>Apr 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2839,24 +2839,24 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>May 1, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Research Internship</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -2871,189 +2871,169 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>May 1, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Ontario, Canada / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>Apr 10, 2026</t>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>Crowdstrike</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>GTM Automation Intern</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Jun 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Anthropic Fellows Program, AI Safety</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Ontario, Canada / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>Apr 10, 2026</t>
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>RBC</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Machine Learning Software Engineer Co-op</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>May 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Software Development Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>https://amazon.jobs/en/jobs/10387163/software-development-engineer-internship-fall-2026-canada</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>Apr 9, 2026</t>
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Diligent Corporation</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>May 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>Tenstorrent</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>IP Product Operations</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Design Verification Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>Feb 4, 2026</t>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Intact</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Data Scientist Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Crowdstrike</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>GTM Automation Intern</t>
+          <t>Application Engineer Co-op</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -3064,24 +3044,24 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Jun 18, 2026</t>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Software Engineer Co-op</t>
+          <t>Data Analyst Intern, Customer Success Operations</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -3092,7 +3072,7 @@
       <c r="E82" s="4" t="inlineStr"/>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>May 23, 2026</t>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-08-16
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$305</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$306</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F305"/>
+  <dimension ref="A1:F306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Engineers and Geoscientists BC</t>
+          <t>CLEAResult</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Information Systems Co-op</t>
+          <t>Energy Efficiency Analyst Co-op</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://egbc.applytojob.com/apply/FYOlZPW8Z5/Information-Systems-Coop</t>
+          <t>https://clearesult.wd1.myworkdayjobs.com/CLEAResult_External_Careers/job/Remote---Canada---BC/Energy-Efficiency-Co-op_R0017820</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Aug 7, 2026</t>
+          <t>Aug 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CLEAResult</t>
+          <t>Engineers and Geoscientists BC</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Energy Efficiency Analyst Co-op</t>
+          <t>Information Systems Co-op</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://clearesult.wd1.myworkdayjobs.com/CLEAResult_External_Careers/job/Remote---Canada---BC/Energy-Efficiency-Co-Op_R0017859</t>
+          <t>https://egbc.applytojob.com/apply/FYOlZPW8Z5/Information-Systems-Coop</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Aug 7, 2026</t>
         </is>
       </c>
     </row>
@@ -2403,17 +2403,17 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Occidental Petroleum</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Process Systems Engineering Co-op, Automation &amp; Data Integration</t>
+          <t>Software Engineering Developer Co-op</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Squamish, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>https://oxy.wd5.myworkdayjobs.com/Corporate/job/Squamish/Process-Systems-Engineering--Automation---Data-Integration---Co-op_JR108371</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000124931443</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2435,17 +2435,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Developer Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000124931443</t>
+          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>May 6, 2026</t>
+          <t>May 1, 2026</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Research Internship</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/8c035d3d-081d-4c8a-914a-72f4efaad254/</t>
+          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2499,17 +2499,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Research Internship</t>
+          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Ontario, Canada / Remote, Canada</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cohere/73bd3e2b-6597-4124-b64b-1e5dbc32e785/</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>May 1, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, ML Systems &amp; Performance</t>
+          <t>Anthropic Fellows Program, AI Safety</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183051008</t>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2563,17 +2563,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Tenstorrent</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Fellows Program, AI Safety</t>
+          <t>IP Product Operations</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Ontario, Canada / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2583,24 +2583,24 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/anthropic/jobs/5183044008</t>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Apr 10, 2026</t>
+          <t>Feb 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Tenstorrent</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>IP Product Operations</t>
+          <t>Forward Deployed Engineering Intern (AI Agent)</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2615,44 +2615,40 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/4530843007</t>
+          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Feb 4, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Cresta</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineering Intern (AI Agent)</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>CLEAResult</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Energy Efficiency Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/cresta/jobs/5106468008</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Feb 2, 2026</t>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
         </is>
       </c>
     </row>
@@ -3275,17 +3271,17 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Occidental Petroleum</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Process Systems Engineering Co-op, Automation &amp; Data Integration</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Squamish, BC</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3296,24 +3292,24 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>May 5, 2026</t>
+          <t>May 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Design Methodology Engineer Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -3336,7 +3332,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Firmware Development Engineer Intern</t>
+          <t>Design Methodology Engineer Intern</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -3364,7 +3360,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Design Emulation Engineer Intern</t>
+          <t>Firmware Development Engineer Intern</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -3387,17 +3383,17 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Diligent Corporation</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Design Emulation Engineer Intern</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -3415,17 +3411,17 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Diligent Corporation</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Design Verification Engineer Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -3436,24 +3432,24 @@
       <c r="E96" s="4" t="inlineStr"/>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>May 4, 2026</t>
+          <t>May 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Data Scientist Intern/Co-op</t>
+          <t>Design Verification Engineer Intern</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3471,12 +3467,12 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Application Engineer Co-op</t>
+          <t>Data Scientist Intern/Co-op</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -3499,17 +3495,17 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Data Analyst Intern, Customer Success Operations</t>
+          <t>Application Engineer Co-op</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3527,17 +3523,17 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Data Analyst Intern, Customer Success Operations</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Burnaby, BC / Oakville, ON</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -3548,7 +3544,7 @@
       <c r="E100" s="4" t="inlineStr"/>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Apr 29, 2026</t>
+          <t>May 4, 2026</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3556,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -3583,12 +3579,12 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -3604,24 +3600,24 @@
       <c r="E102" s="4" t="inlineStr"/>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Apr 24, 2026</t>
+          <t>Apr 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Stryker</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Systems R&amp;D Engineer Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3632,24 +3628,24 @@
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Apr 17, 2026</t>
+          <t>Apr 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Stryker</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern Fall</t>
+          <t>Systems R&amp;D Engineer Co-op</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -3667,17 +3663,17 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Software Engineer Intern Fall</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -3723,12 +3719,12 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Revvity</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Test and Manufacturing Intern</t>
+          <t>Full-Stack AI Developer Intern</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -3744,24 +3740,24 @@
       <c r="E107" s="4" t="inlineStr"/>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>Apr 16, 2026</t>
+          <t>Apr 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>OpusClip</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>AI Product Manager Intern</t>
+          <t>Test and Manufacturing Intern</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -3772,19 +3768,19 @@
       <c r="E108" s="4" t="inlineStr"/>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Apr 14, 2026</t>
+          <t>Apr 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>OpusClip</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Product Management Intern</t>
+          <t>AI Product Manager Intern</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -3800,19 +3796,19 @@
       <c r="E109" s="4" t="inlineStr"/>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>Apr 11, 2026</t>
+          <t>Apr 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Intern/Co-op - Internal AI Operations</t>
+          <t>Product Management Intern</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -3828,19 +3824,19 @@
       <c r="E110" s="4" t="inlineStr"/>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>Apr 10, 2026</t>
+          <t>Apr 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Intern/Co-op - Internal AI Operations</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -3856,24 +3852,24 @@
       <c r="E111" s="4" t="inlineStr"/>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>Apr 9, 2026</t>
+          <t>Apr 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>BMW Group</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -3884,24 +3880,24 @@
       <c r="E112" s="4" t="inlineStr"/>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>Apr 7, 2026</t>
+          <t>Apr 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>BMW Group</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>AI / Machine Learning Intern</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -3919,17 +3915,17 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Diligent Corporation</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>AI / Machine Learning Intern</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -3940,24 +3936,24 @@
       <c r="E114" s="4" t="inlineStr"/>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Apr 1, 2026</t>
+          <t>Apr 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Diligent Corporation</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Product Management Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -3968,24 +3964,24 @@
       <c r="E115" s="4" t="inlineStr"/>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Mar 31, 2026</t>
+          <t>Apr 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>DotDash Meredith</t>
+          <t>Fortinet</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Product Management Intern</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Remote</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -4003,17 +3999,17 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>DotDash Meredith</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Software Developer. Web/Cloud Application</t>
+          <t>Data Engineering Intern</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Edmonton, AB / Remote</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -4024,24 +4020,24 @@
       <c r="E117" s="4" t="inlineStr"/>
       <c r="F117" s="4" t="inlineStr">
         <is>
-          <t>Mar 26, 2026</t>
+          <t>Mar 31, 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern ML AI, Fall 2026</t>
+          <t>Software Developer. Web/Cloud Application</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -4052,24 +4048,24 @@
       <c r="E118" s="4" t="inlineStr"/>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Mar 24, 2026</t>
+          <t>Mar 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack AI Developer Intern</t>
+          <t>Software Engineer Intern ML AI, Fall 2026</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -4080,24 +4076,24 @@
       <c r="E119" s="4" t="inlineStr"/>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>Mar 23, 2026</t>
+          <t>Mar 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Revvity</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer, The Coalition: Intern Opportunities</t>
+          <t>Full-Stack AI Developer Intern</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -4108,24 +4104,24 @@
       <c r="E120" s="4" t="inlineStr"/>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>Mar 20, 2026</t>
+          <t>Mar 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Cloud Architecture</t>
+          <t>Software Engineer, The Coalition: Intern Opportunities</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -4136,24 +4132,24 @@
       <c r="E121" s="4" t="inlineStr"/>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>Mar 18, 2026</t>
+          <t>Mar 20, 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>DotDash Meredith</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Transaction Tooling Intern</t>
+          <t>Software Engineering Intern, Cloud Architecture</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -4171,17 +4167,17 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>DotDash Meredith</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer. Intern Opportunities for University Students</t>
+          <t>Transaction Tooling Intern</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -4199,17 +4195,17 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>People Inc</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer. Intern Opportunities for University Students</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
@@ -4220,24 +4216,24 @@
       <c r="E124" s="4" t="inlineStr"/>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>Mar 13, 2026</t>
+          <t>Mar 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>Canadian Tire</t>
+          <t>People Inc</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Innovation &amp; Testing Student</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -4260,7 +4256,7 @@
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Apparel Design Student</t>
+          <t>Innovation &amp; Testing Student</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
@@ -4283,17 +4279,17 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>WSP</t>
+          <t>Canadian Tire</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Web Developer Intern</t>
+          <t>Apparel Design Student</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -4311,17 +4307,17 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>WSP</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Health Informatics Intern</t>
+          <t>Web Developer Intern</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -4332,24 +4328,24 @@
       <c r="E128" s="4" t="inlineStr"/>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>Mar 10, 2026</t>
+          <t>Mar 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Data Enablement</t>
+          <t>Health Informatics Intern</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -4360,24 +4356,24 @@
       <c r="E129" s="4" t="inlineStr"/>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>Mar 9, 2026</t>
+          <t>Mar 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Juniper Square</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer Intern</t>
+          <t>Data Enablement</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -4395,17 +4391,17 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>AssetWorks</t>
+          <t>Juniper Square</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>AI Engineer Intern</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -4423,17 +4419,17 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Cohere</t>
+          <t>AssetWorks</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Safety Research Intern</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -4451,17 +4447,17 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
+          <t>Safety Research Intern</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -4472,24 +4468,24 @@
       <c r="E133" s="4" t="inlineStr"/>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>Mar 6, 2026</t>
+          <t>Mar 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Data Engineer</t>
+          <t>Engineering/Development Intern/Co-op, Fall 2026</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -4507,17 +4503,17 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>GIS Intern, Geospatial Services</t>
+          <t>Software Engineering Intern, Data Engineer</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -4528,24 +4524,24 @@
       <c r="E135" s="4" t="inlineStr"/>
       <c r="F135" s="4" t="inlineStr">
         <is>
-          <t>Mar 4, 2026</t>
+          <t>Mar 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Developer Co-op</t>
+          <t>GIS Intern, Geospatial Services</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Waterloo, ON / Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
@@ -4556,24 +4552,24 @@
       <c r="E136" s="4" t="inlineStr"/>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>Mar 3, 2026</t>
+          <t>Mar 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
+          <t>Developer Co-op</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Waterloo, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
@@ -4584,7 +4580,7 @@
       <c r="E137" s="4" t="inlineStr"/>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>Mar 2, 2026</t>
+          <t>Mar 3, 2026</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4592,7 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Full-Stack Engineer Intern, Fall 2026</t>
+          <t>Software Engineer Intern, AI Enablement, Fall 2026</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
@@ -4624,7 +4620,7 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern, Fall 2026</t>
+          <t>Full-Stack Engineer Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
@@ -4647,17 +4643,17 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Co-op Java Developer, Summer 2026</t>
+          <t>Frontend Engineering Intern, Fall 2026</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -4668,7 +4664,7 @@
       <c r="E140" s="4" t="inlineStr"/>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>Feb 27, 2026</t>
+          <t>Mar 2, 2026</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4681,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -4703,17 +4699,17 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>User Research Co-op</t>
+          <t>Co-op Java Developer, Summer 2026</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
@@ -4724,19 +4720,19 @@
       <c r="E142" s="4" t="inlineStr"/>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>Feb 26, 2026</t>
+          <t>Feb 27, 2026</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Localization Software Developer, Co-Op</t>
+          <t>User Research Co-op</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -4752,24 +4748,24 @@
       <c r="E143" s="4" t="inlineStr"/>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>Feb 25, 2026</t>
+          <t>Feb 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Localization Software Developer, Co-Op</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
@@ -4787,12 +4783,12 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>Correlation One</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
@@ -4815,17 +4811,17 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>Kabam</t>
+          <t>Correlation One</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op (Systems)</t>
+          <t>Lead Instructor: Data Analytics, Apprenticeship Program</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
@@ -4836,24 +4832,24 @@
       <c r="E146" s="4" t="inlineStr"/>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>Feb 24, 2026</t>
+          <t>Feb 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>Kabam</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
+          <t>Software Engineer Co-op (Systems)</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
@@ -4864,19 +4860,19 @@
       <c r="E147" s="4" t="inlineStr"/>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>Feb 19, 2026</t>
+          <t>Feb 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Junior Engineer, Co-op/Internship, Electronic Trading Infrastructure, Summer 2026</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -4899,17 +4895,17 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>Critical Mass</t>
+          <t>Jonas Software</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Development Intern</t>
+          <t>Jonas Summer Internship – Various Departments</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -4927,17 +4923,17 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Critical Mass</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Automation Development Student</t>
+          <t>Development Intern</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Acheson, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -4948,24 +4944,24 @@
       <c r="E150" s="4" t="inlineStr"/>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>Feb 18, 2026</t>
+          <t>Feb 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Data Analytics &amp; Automation Development Student</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB / Acheson, AB</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -4983,17 +4979,17 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>Sanctuary AI</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
@@ -5011,17 +5007,17 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Sanctuary AI</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Automation Consulting Intern/Co-op</t>
+          <t>Machine Learning Research Intern, Reinforcement/Imitation Learning</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
@@ -5032,24 +5028,24 @@
       <c r="E153" s="4" t="inlineStr"/>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>Feb 17, 2026</t>
+          <t>Feb 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>CAE</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>C-MAT-100 Engineering Intern</t>
+          <t>Automation Consulting Intern/Co-op</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Moose Jaw, SK</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
@@ -5060,24 +5056,24 @@
       <c r="E154" s="4" t="inlineStr"/>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>Feb 16, 2026</t>
+          <t>Feb 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>CAE</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Application Engineer Test Intern</t>
+          <t>C-MAT-100 Engineering Intern</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Moose Jaw, SK</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
@@ -5095,17 +5091,17 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>RSM</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Business Intelligence Consulting Associate - Fall 2026</t>
+          <t>Application Engineer Test Intern</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
@@ -5116,24 +5112,24 @@
       <c r="E156" s="4" t="inlineStr"/>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>Feb 13, 2026</t>
+          <t>Feb 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>RSM</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Student Digital Systems</t>
+          <t>Business Intelligence Consulting Associate - Fall 2026</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -5144,24 +5140,24 @@
       <c r="E157" s="4" t="inlineStr"/>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>Feb 11, 2026</t>
+          <t>Feb 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Student Digital Systems</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
@@ -5172,24 +5168,24 @@
       <c r="E158" s="4" t="inlineStr"/>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>Feb 10, 2026</t>
+          <t>Feb 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Design Methodology Engineering Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
@@ -5212,7 +5208,7 @@
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>System Simulation Engineer Intern</t>
+          <t>Design Methodology Engineering Intern</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -5235,17 +5231,17 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>Fullscript</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>System Simulation Engineer Intern</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Ottawa, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
@@ -5263,17 +5259,17 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Fullscript</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
@@ -5284,19 +5280,19 @@
       <c r="E162" s="4" t="inlineStr"/>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>Feb 9, 2026</t>
+          <t>Feb 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Applied Research Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -5319,17 +5315,17 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Intern, Dto, Enterprise Analytics</t>
+          <t>Applied Research Intern</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
@@ -5352,7 +5348,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
+          <t>Intern, Dto, Enterprise Analytics</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -5380,7 +5376,7 @@
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Intern, Data &amp; Integrations</t>
+          <t>Business Technology Solutions, Enterprise Resource Planning Implementation</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -5403,12 +5399,12 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Design Validation Intern/Co-op</t>
+          <t>Intern, Data &amp; Integrations</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -5431,17 +5427,17 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>Mikata Health</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Data Science Intern</t>
+          <t>Design Validation Intern/Co-op</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
@@ -5459,17 +5455,17 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Instacart</t>
+          <t>Mikata Health</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Data Science PhD Intern</t>
+          <t>Healthcare Data Science Intern</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
@@ -5480,19 +5476,19 @@
       <c r="E169" s="4" t="inlineStr"/>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>Feb 5, 2026</t>
+          <t>Feb 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Instacart</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Client Secrets Management</t>
+          <t>Data Science PhD Intern</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -5508,24 +5504,24 @@
       <c r="E170" s="4" t="inlineStr"/>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>Feb 3, 2026</t>
+          <t>Feb 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Developer Intern - Client Secrets Management</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Richmond Hill, ON</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
@@ -5536,24 +5532,24 @@
       <c r="E171" s="4" t="inlineStr"/>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>Feb 2, 2026</t>
+          <t>Feb 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Data Intern - Enterprise Analytics</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond Hill, ON</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
@@ -5571,17 +5567,17 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Veralto</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning Co-Op Intern</t>
+          <t>Data Intern - Enterprise Analytics</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
@@ -5592,24 +5588,24 @@
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>Feb 1, 2026</t>
+          <t>Feb 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Veralto</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Knox</t>
+          <t>Machine Learning Co-Op Intern</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -5620,7 +5616,7 @@
       <c r="E174" s="4" t="inlineStr"/>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>Jan 30, 2026</t>
+          <t>Feb 1, 2026</t>
         </is>
       </c>
     </row>
@@ -5632,7 +5628,7 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Trust Platforms</t>
+          <t>Developer Intern - Knox</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -5660,7 +5656,7 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Extension Excellence</t>
+          <t>Developer Intern - Trust Platforms</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
@@ -5688,7 +5684,7 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Insights</t>
+          <t>Developer Intern - Extension Excellence</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -5716,7 +5712,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement</t>
+          <t>Developer Intern - Insights</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
@@ -5744,7 +5740,7 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Device Security</t>
+          <t>Developer Intern - Platform Advancement</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -5772,7 +5768,7 @@
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Billing &amp; Payments</t>
+          <t>Developer Intern - Device Security</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
@@ -5800,7 +5796,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Data &amp; Access</t>
+          <t>Developer Intern - Billing &amp; Payments</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -5823,17 +5819,17 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>Ovintiv</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Student Engineer</t>
+          <t>Developer Intern - Data &amp; Access</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
@@ -5851,17 +5847,17 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Voldex</t>
+          <t>Ovintiv</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Game Developer Intern</t>
+          <t>Student Engineer</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
@@ -5872,19 +5868,19 @@
       <c r="E183" s="4" t="inlineStr"/>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Jan 29, 2026</t>
+          <t>Jan 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>GE Healthcare</t>
+          <t>Voldex</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>Field Service Apprentice</t>
+          <t>Game Developer Intern</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
@@ -5900,24 +5896,24 @@
       <c r="E184" s="4" t="inlineStr"/>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>Jan 28, 2026</t>
+          <t>Jan 29, 2026</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>GE Healthcare</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-Op</t>
+          <t>Field Service Apprentice</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
@@ -5935,17 +5931,17 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern/Co-op</t>
+          <t>Software Engineer Co-Op</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
@@ -5956,24 +5952,24 @@
       <c r="E186" s="4" t="inlineStr"/>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>Jan 26, 2026</t>
+          <t>Jan 28, 2026</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>BC Pensions</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>Application Developer Intern/Co-op</t>
+          <t>Software Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
@@ -5991,17 +5987,17 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>BC Pensions</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>Support Enablement Engineer Intern</t>
+          <t>Application Developer Intern/Co-op</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
@@ -6012,19 +6008,19 @@
       <c r="E188" s="4" t="inlineStr"/>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>Jan 23, 2026</t>
+          <t>Jan 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Intern Full Stack Developer</t>
+          <t>Support Enablement Engineer Intern</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -6047,12 +6043,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Allstate Insurance Company</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>Data Governance Intern/Co-op</t>
+          <t>Intern Full Stack Developer</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -6068,7 +6064,7 @@
       <c r="E190" s="4" t="inlineStr"/>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>Jan 22, 2026</t>
+          <t>Jan 23, 2026</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6076,7 @@
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Provincial Product Analyst Co-op</t>
+          <t>Data Governance Intern/Co-op</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -6103,17 +6099,17 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Allstate Insurance Company</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern - Summer 2026</t>
+          <t>Provincial Product Analyst Co-op</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
@@ -6124,7 +6120,7 @@
       <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>Jan 21, 2026</t>
+          <t>Jan 22, 2026</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6132,7 @@
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern - Summer 2026</t>
+          <t>Production Engineering Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -6164,7 +6160,7 @@
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Graduate Production Engineer Research Intern</t>
+          <t>Studio Talent Group Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -6192,7 +6188,7 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Technical Assistant Intern - Summer 2026</t>
+          <t>Graduate Production Engineer Research Intern</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -6215,17 +6211,17 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>BMO</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Co-op/Internship</t>
+          <t>Technical Assistant Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
@@ -6236,19 +6232,19 @@
       <c r="E196" s="4" t="inlineStr"/>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>Jan 19, 2026</t>
+          <t>Jan 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Bank of Montreal</t>
+          <t>BMO</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Developer – Co-op/Internship</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -6271,17 +6267,17 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>Bank of Montreal</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>Engineering Intern</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
@@ -6292,24 +6288,24 @@
       <c r="E198" s="4" t="inlineStr"/>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>Jan 17, 2026</t>
+          <t>Jan 19, 2026</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>The Boeing Company</t>
+          <t>Boomi</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering Intern</t>
+          <t>Engineering Intern</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
@@ -6320,7 +6316,7 @@
       <c r="E199" s="4" t="inlineStr"/>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>Jan 16, 2026</t>
+          <t>Jan 17, 2026</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6328,7 @@
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Data Engineering Intern</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -6360,7 +6356,7 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>Data Science Business Operations Intern</t>
+          <t>Data Science Intern</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -6383,17 +6379,17 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Harris Computer</t>
+          <t>The Boeing Company</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>Systems Analyst</t>
+          <t>Data Science Business Operations Intern</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
@@ -6411,12 +6407,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Nokia</t>
+          <t>Harris Computer</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>AI/ML Coop/Intern</t>
+          <t>Systems Analyst</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -6439,17 +6435,17 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>Enbridge</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>SharePoint &amp; Document Management Support - Summer Student</t>
+          <t>AI/ML Coop/Intern</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
@@ -6467,17 +6463,17 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Enbridge</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>Game Creation SW Engineer Intern</t>
+          <t>SharePoint &amp; Document Management Support - Summer Student</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -6488,24 +6484,24 @@
       <c r="E205" s="4" t="inlineStr"/>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>Jan 15, 2026</t>
+          <t>Jan 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
+          <t>Game Creation SW Engineer Intern</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
@@ -6528,7 +6524,7 @@
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Enterprise Solutions Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -6551,17 +6547,17 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
@@ -6572,19 +6568,19 @@
       <c r="E208" s="4" t="inlineStr"/>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>Jan 13</t>
+          <t>Jan 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer - Internship Opportunities</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -6600,24 +6596,24 @@
       <c r="E209" s="4" t="inlineStr"/>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>Jan 12</t>
+          <t>Jan 13</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineering Intern</t>
+          <t>Software Engineer - Internship Opportunities</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
@@ -6628,24 +6624,24 @@
       <c r="E210" s="4" t="inlineStr"/>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>Jan 9</t>
+          <t>Jan 12</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>Triton Compiler Engineering Intern</t>
+          <t>Systems Software Engineering Intern</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Remote in Canada</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
@@ -6663,17 +6659,17 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - Co-op - Full Stack</t>
+          <t>Triton Compiler Engineering Intern</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
@@ -6696,7 +6692,7 @@
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
+          <t>Software Developer - Co-op - Full Stack</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
@@ -6724,7 +6720,7 @@
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>Software Developer - C++ - Co-op</t>
+          <t>Software Developer (Cloud Infrastructure) - Co-Op</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
@@ -6747,12 +6743,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer - C++ - Co-op</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -6775,17 +6771,17 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op/Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
@@ -6796,24 +6792,24 @@
       <c r="E216" s="4" t="inlineStr"/>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t>Jan 8</t>
+          <t>Jan 9</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
@@ -6831,7 +6827,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -6852,14 +6848,14 @@
       <c r="E218" s="4" t="inlineStr"/>
       <c r="F218" s="4" t="inlineStr">
         <is>
-          <t>Jan 7</t>
+          <t>Jan 8</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>ATPCO</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
@@ -6880,24 +6876,24 @@
       <c r="E219" s="4" t="inlineStr"/>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>Jan 6</t>
+          <t>Jan 7</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>ATPCO</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern/Co-op - Oracle APEX</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
@@ -6908,24 +6904,24 @@
       <c r="E220" s="4" t="inlineStr"/>
       <c r="F220" s="4" t="inlineStr">
         <is>
-          <t>Jan 5</t>
+          <t>Jan 6</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Intern/Co-op - Oracle APEX</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
@@ -6943,17 +6939,17 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>BDC</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
@@ -6971,17 +6967,17 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>BDC</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
+          <t>SUMMER STUDENTS 2026 - INFORMATION TECHNOLOGY</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Montreal, QC / Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
@@ -6992,7 +6988,7 @@
       <c r="E223" s="4" t="inlineStr"/>
       <c r="F223" s="4" t="inlineStr">
         <is>
-          <t>Dec 20</t>
+          <t>Jan 5</t>
         </is>
       </c>
     </row>
@@ -7004,12 +7000,12 @@
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
+          <t>Entry Level Technology Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
+          <t>Calgary, AB / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
@@ -7027,17 +7023,17 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Accenture</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern - Echo</t>
+          <t>Entry Level Consulting Analyst Development Program - Summer Analyst (Intern)</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Calgary, AB / Vancouver, BC / Ottawa, ON / Toronto, ON / Montreal, QC</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
@@ -7048,24 +7044,24 @@
       <c r="E225" s="4" t="inlineStr"/>
       <c r="F225" s="4" t="inlineStr">
         <is>
-          <t>Dec 18</t>
+          <t>Dec 20</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer Intern - Echo</t>
         </is>
       </c>
       <c r="C226" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr">
@@ -7076,24 +7072,24 @@
       <c r="E226" s="4" t="inlineStr"/>
       <c r="F226" s="4" t="inlineStr">
         <is>
-          <t>Dec 17</t>
+          <t>Dec 18</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - AI/ML QVS</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
@@ -7104,24 +7100,24 @@
       <c r="E227" s="4" t="inlineStr"/>
       <c r="F227" s="4" t="inlineStr">
         <is>
-          <t>Dec 15</t>
+          <t>Dec 17</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>RBC Borealis - Machine Learning Software Engineer</t>
+          <t>Software Engineer Intern - AI/ML QVS</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
@@ -7132,24 +7128,24 @@
       <c r="E228" s="4" t="inlineStr"/>
       <c r="F228" s="4" t="inlineStr">
         <is>
-          <t>Dec 12</t>
+          <t>Dec 15</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Applications - Summer 2026</t>
+          <t>RBC Borealis - Machine Learning Software Engineer</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Calgary, AL / Vancouver, BC</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
@@ -7172,7 +7168,7 @@
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
+          <t>Software Engineering Intern, Applications - Summer 2026</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
@@ -7195,12 +7191,12 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>Production Engineering Intern</t>
+          <t>Software Engineering Intern, Connected Systems - Summer 2026</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -7228,7 +7224,7 @@
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>Studio Talent Group Intern</t>
+          <t>Production Engineering Intern</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -7244,19 +7240,19 @@
       <c r="E232" s="4" t="inlineStr"/>
       <c r="F232" s="4" t="inlineStr">
         <is>
-          <t>Dec 11</t>
+          <t>Dec 12</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>DataVisor</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>Backend Software Engineer Internship</t>
+          <t>Studio Talent Group Intern</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -7272,24 +7268,24 @@
       <c r="E233" s="4" t="inlineStr"/>
       <c r="F233" s="4" t="inlineStr">
         <is>
-          <t>Dec 10</t>
+          <t>Dec 11</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>DataVisor</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op</t>
+          <t>Backend Software Engineer Internship</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>Kitchener, ON / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
@@ -7307,17 +7303,17 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern - Summer 2026</t>
+          <t>Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Ottawa, ON / Calgary, AB / Vancouver, BC / Victoria, BC</t>
+          <t>Kitchener, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
@@ -7328,24 +7324,24 @@
       <c r="E235" s="4" t="inlineStr"/>
       <c r="F235" s="4" t="inlineStr">
         <is>
-          <t>Dec 9</t>
+          <t>Dec 10</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>Standard Aero</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>Computer Engineering Intern - TFE Service Team</t>
+          <t>Software Development Engineer Intern - Summer 2026</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Toronto, ON / Ottawa, ON / Calgary, AB / Vancouver, BC / Victoria, BC</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
@@ -7356,24 +7352,24 @@
       <c r="E236" s="4" t="inlineStr"/>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Dec 1</t>
+          <t>Dec 9</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>Ticketmaster</t>
+          <t>Standard Aero</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Computer Engineering Intern - TFE Service Team</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
@@ -7384,24 +7380,24 @@
       <c r="E237" s="4" t="inlineStr"/>
       <c r="F237" s="4" t="inlineStr">
         <is>
-          <t>Nov 26</t>
+          <t>Dec 1</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Ticketmaster</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>Systems Software Engineer Intern/Co-op</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
@@ -7412,24 +7408,24 @@
       <c r="E238" s="4" t="inlineStr"/>
       <c r="F238" s="4" t="inlineStr">
         <is>
-          <t>Nov 15</t>
+          <t>Nov 26</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>Volaris Group</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Systems Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>Mississauga, ON, Canada / Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr">
@@ -7440,24 +7436,24 @@
       <c r="E239" s="4" t="inlineStr"/>
       <c r="F239" s="4" t="inlineStr">
         <is>
-          <t>Nov 14</t>
+          <t>Nov 15</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Volaris Group</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>Co-Op/Intern – Software Development – Winter 2026</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Calgary, AB / Vancouver, BC</t>
+          <t>Mississauga, ON, Canada / Remote in Canada</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
@@ -7468,24 +7464,24 @@
       <c r="E240" s="4" t="inlineStr"/>
       <c r="F240" s="4" t="inlineStr">
         <is>
-          <t>Nov 13</t>
+          <t>Nov 14</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Connected Systems, Summer 2026</t>
+          <t>Co-Op/Intern – Software Development – Winter 2026</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Calgary, AB / Vancouver, BC</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
@@ -7508,7 +7504,7 @@
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>Software Automation Engineering Intern, Summer 2026</t>
+          <t>Software Engineering Intern, Connected Systems, Summer 2026</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr">
@@ -7531,12 +7527,12 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>Transcarent</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Software Engineer Intern</t>
+          <t>Software Automation Engineering Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr">
@@ -7552,24 +7548,24 @@
       <c r="E243" s="4" t="inlineStr"/>
       <c r="F243" s="4" t="inlineStr">
         <is>
-          <t>Nov 7</t>
+          <t>Nov 13</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>Valsoft Corporation</t>
+          <t>Transcarent</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
+          <t>Full Stack Software Engineer Intern</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
@@ -7580,7 +7576,7 @@
       <c r="E244" s="4" t="inlineStr"/>
       <c r="F244" s="4" t="inlineStr">
         <is>
-          <t>Nov 5</t>
+          <t>Nov 7</t>
         </is>
       </c>
     </row>
@@ -7592,7 +7588,7 @@
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer Intern – AI Engagement Portal</t>
+          <t>Full Stack Development Intern – Agentic AI &amp; Cloud-Native</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
@@ -7615,17 +7611,17 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Valsoft Corporation</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Full Stack Developer Intern – AI Engagement Portal</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
@@ -7643,12 +7639,12 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Applications, Infotainment &amp; Mobile</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
@@ -7671,12 +7667,12 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Software Engineering Intern, Applications, Infotainment &amp; Mobile</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr">
@@ -7692,24 +7688,24 @@
       <c r="E248" s="4" t="inlineStr"/>
       <c r="F248" s="4" t="inlineStr">
         <is>
-          <t>Nov 4</t>
+          <t>Nov 5</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>Intern - Software Developer</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>Montreal, QC, Canada (Remote in Canada)</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
@@ -7727,17 +7723,17 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>Developer, RBC Amplify 2026</t>
+          <t>Intern - Software Developer</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Montreal, QC, Canada (Remote in Canada)</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr">
@@ -7748,7 +7744,7 @@
       <c r="E250" s="4" t="inlineStr"/>
       <c r="F250" s="4" t="inlineStr">
         <is>
-          <t>Nov 3</t>
+          <t>Nov 4</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7761,7 @@
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr">
@@ -7783,17 +7779,17 @@
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>Global Relay</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>Frontend Software Developer Co-op (React.js)</t>
+          <t>Developer, RBC Amplify 2026</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
@@ -7804,7 +7800,7 @@
       <c r="E252" s="4" t="inlineStr"/>
       <c r="F252" s="4" t="inlineStr">
         <is>
-          <t>Oct 30</t>
+          <t>Nov 3</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7812,7 @@
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
+          <t>Frontend Software Developer Co-op (React.js)</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
@@ -7849,7 +7845,7 @@
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>Kelowna, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr">
@@ -7867,17 +7863,17 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>Rivian</t>
+          <t>Global Relay</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
+          <t>Software Development Engineer in Test (SDET)- Co-op - Winter 2026</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Kelowna, BC</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
@@ -7888,19 +7884,19 @@
       <c r="E255" s="4" t="inlineStr"/>
       <c r="F255" s="4" t="inlineStr">
         <is>
-          <t>Oct 29</t>
+          <t>Oct 30</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>Dialpad</t>
+          <t>Rivian</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op, Front End</t>
+          <t>Software Engineering Internships (Winter 2026 Co-Op Program)</t>
         </is>
       </c>
       <c r="C256" s="4" t="inlineStr">
@@ -7928,7 +7924,7 @@
       </c>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Fullstack</t>
+          <t>Software Engineer Co-op, Front End</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr">
@@ -7956,7 +7952,7 @@
       </c>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>Co-op Software Engineer, Backend</t>
+          <t>Co-op Software Engineer, Fullstack</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr">
@@ -7979,17 +7975,17 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Dialpad</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Summer 2026</t>
+          <t>Co-op Software Engineer, Backend</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
@@ -8000,24 +7996,24 @@
       <c r="E259" s="4" t="inlineStr"/>
       <c r="F259" s="4" t="inlineStr">
         <is>
-          <t>Oct 27</t>
+          <t>Oct 29</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Engineer Internship – Summer 2026</t>
         </is>
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC - Toronto, ON - Ottawa, ON - Calgary, AB - Victoria, BC - Winnipeg, MB</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
@@ -8028,19 +8024,19 @@
       <c r="E260" s="4" t="inlineStr"/>
       <c r="F260" s="4" t="inlineStr">
         <is>
-          <t>Oct 24</t>
+          <t>Oct 27</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
@@ -8056,7 +8052,7 @@
       <c r="E261" s="4" t="inlineStr"/>
       <c r="F261" s="4" t="inlineStr">
         <is>
-          <t>Oct 23</t>
+          <t>Oct 24</t>
         </is>
       </c>
     </row>
@@ -8068,7 +8064,7 @@
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>Agile Test Developer Intern</t>
+          <t>Cloud ERP Solution Adoption Data Analyst Intern</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr">
@@ -8084,7 +8080,7 @@
       <c r="E262" s="4" t="inlineStr"/>
       <c r="F262" s="4" t="inlineStr">
         <is>
-          <t>Oct 22</t>
+          <t>Oct 23</t>
         </is>
       </c>
     </row>
@@ -8096,7 +8092,7 @@
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>Cloud Engineer Intern</t>
+          <t>Agile Test Developer Intern</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
@@ -8112,7 +8108,7 @@
       <c r="E263" s="4" t="inlineStr"/>
       <c r="F263" s="4" t="inlineStr">
         <is>
-          <t>Oct 20</t>
+          <t>Oct 22</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8120,7 @@
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>AI Software Developer Intern</t>
+          <t>Cloud Engineer Intern</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
@@ -8140,24 +8136,24 @@
       <c r="E264" s="4" t="inlineStr"/>
       <c r="F264" s="4" t="inlineStr">
         <is>
-          <t>Oct 18</t>
+          <t>Oct 20</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>The Athletic</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>Engineering Student Intern, Summer 2026</t>
+          <t>AI Software Developer Intern</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
@@ -8168,24 +8164,24 @@
       <c r="E265" s="4" t="inlineStr"/>
       <c r="F265" s="4" t="inlineStr">
         <is>
-          <t>Oct 17</t>
+          <t>Oct 18</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>The Athletic</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>SAP Analytics Cloud Security Engineer Intern</t>
+          <t>Engineering Student Intern, Summer 2026</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
@@ -8196,24 +8192,24 @@
       <c r="E266" s="4" t="inlineStr"/>
       <c r="F266" s="4" t="inlineStr">
         <is>
-          <t>Oct 16</t>
+          <t>Oct 17</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>Journal Technologies</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>Junior Software Developer Co-op</t>
+          <t>SAP Analytics Cloud Security Engineer Intern</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
@@ -8231,17 +8227,17 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>Canada Life</t>
+          <t>Journal Technologies</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Student Position)</t>
+          <t>Junior Software Developer Co-op</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Winnipeg, MB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
@@ -8252,24 +8248,24 @@
       <c r="E268" s="4" t="inlineStr"/>
       <c r="F268" s="4" t="inlineStr">
         <is>
-          <t>Oct 15</t>
+          <t>Oct 16</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Canada Life</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>Full-stack Engineering Intern</t>
+          <t>Software Developer (Student Position)</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Toronto, ON / Winnipeg, MB</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
@@ -8280,7 +8276,7 @@
       <c r="E269" s="4" t="inlineStr"/>
       <c r="F269" s="4" t="inlineStr">
         <is>
-          <t>Oct 13</t>
+          <t>Oct 15</t>
         </is>
       </c>
     </row>
@@ -8292,7 +8288,7 @@
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>Backend Engineering Intern</t>
+          <t>Full-stack Engineering Intern</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr">
@@ -8320,7 +8316,7 @@
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>Frontend Engineering Intern</t>
+          <t>Backend Engineering Intern</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
@@ -8343,17 +8339,17 @@
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern</t>
+          <t>Frontend Engineering Intern</t>
         </is>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr">
@@ -8364,19 +8360,19 @@
       <c r="E272" s="4" t="inlineStr"/>
       <c r="F272" s="4" t="inlineStr">
         <is>
-          <t>Oct 10</t>
+          <t>Oct 13</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>Seaspan</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>Intern – Digital Ship</t>
+          <t>Software Development Intern</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
@@ -8392,24 +8388,24 @@
       <c r="E273" s="4" t="inlineStr"/>
       <c r="F273" s="4" t="inlineStr">
         <is>
-          <t>Oct 8</t>
+          <t>Oct 10</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>Ada</t>
+          <t>Seaspan</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Intern – Digital Ship</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
@@ -8420,24 +8416,24 @@
       <c r="E274" s="4" t="inlineStr"/>
       <c r="F274" s="4" t="inlineStr">
         <is>
-          <t>Oct 7</t>
+          <t>Oct 8</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Ada</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – Sports Technology</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
@@ -8448,7 +8444,7 @@
       <c r="E275" s="4" t="inlineStr"/>
       <c r="F275" s="4" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 7</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8456,7 @@
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – UFC</t>
+          <t>Software Engineer Intern – Sports Technology</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr">
@@ -8483,17 +8479,17 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>1Password</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Stateful Systems - Winter 2026</t>
+          <t>Software Engineer Intern – UFC</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
@@ -8504,7 +8500,7 @@
       <c r="E277" s="4" t="inlineStr"/>
       <c r="F277" s="4" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 6</t>
         </is>
       </c>
     </row>
@@ -8516,7 +8512,7 @@
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Release Engineering - Winter 2026</t>
+          <t>Developer Intern - Stateful Systems - Winter 2026</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
@@ -8544,7 +8540,7 @@
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Platform Advancement - Winter 2026</t>
+          <t>Developer Intern - Release Engineering - Winter 2026</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
@@ -8572,7 +8568,7 @@
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Frameworks - Winter 2026</t>
+          <t>Developer Intern - Platform Advancement - Winter 2026</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
@@ -8600,7 +8596,7 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
+          <t>Developer Intern - Frameworks - Winter 2026</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -8628,7 +8624,7 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern - App Launcher - Winter 2026</t>
+          <t>Developer Intern - Enterprise Ready - Winter 2026</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
@@ -8651,17 +8647,17 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>Online Software Engineer Co-op</t>
+          <t>Developer Intern - App Launcher - Winter 2026</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
@@ -8672,24 +8668,24 @@
       <c r="E283" s="4" t="inlineStr"/>
       <c r="F283" s="4" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 5</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Internship – Winter 2026</t>
+          <t>Online Software Engineer Co-op</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
@@ -8700,24 +8696,24 @@
       <c r="E284" s="4" t="inlineStr"/>
       <c r="F284" s="4" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 4</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
+          <t>Software Development Engineer Internship – Winter 2026</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC / Toronto, ON / Winnipeg, MB / Victoria, BC / Ottawa, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
@@ -8728,7 +8724,7 @@
       <c r="E285" s="4" t="inlineStr"/>
       <c r="F285" s="4" t="inlineStr">
         <is>
-          <t>Oct 2</t>
+          <t>Oct 3</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8736,7 @@
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern – NHL</t>
+          <t>C++ Software Engineer Intern/Co-op – UI Tech Stack</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
@@ -8768,7 +8764,7 @@
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
+          <t>Software Engineer Intern – NHL</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
@@ -8791,12 +8787,12 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Software Developer – Front-end Co-Op</t>
+          <t>Software Engineer Intern/Co-op - Client Software Engineering</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr">
@@ -8812,24 +8808,24 @@
       <c r="E288" s="4" t="inlineStr"/>
       <c r="F288" s="4" t="inlineStr">
         <is>
-          <t>Oct 1</t>
+          <t>Oct 2</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>Geotab</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Software Development Intern – Multiple Teams</t>
+          <t>Software Developer – Front-end Co-Op</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -8840,24 +8836,24 @@
       <c r="E289" s="4" t="inlineStr"/>
       <c r="F289" s="4" t="inlineStr">
         <is>
-          <t>Sep 23</t>
+          <t>Oct 1</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>Pason</t>
+          <t>Geotab</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Datahub)</t>
+          <t>Software Development Intern – Multiple Teams</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
@@ -8868,7 +8864,7 @@
       <c r="E290" s="4" t="inlineStr"/>
       <c r="F290" s="4" t="inlineStr">
         <is>
-          <t>Sep 18</t>
+          <t>Sep 23</t>
         </is>
       </c>
     </row>
@@ -8880,7 +8876,7 @@
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Quality Assurance)</t>
+          <t>Software Developer Intern (Datahub)</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
@@ -8908,7 +8904,7 @@
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern (Enterprise Applications)</t>
+          <t>Software Developer Intern (Quality Assurance)</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
@@ -8931,12 +8927,12 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Pason</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern/ Co-op</t>
+          <t>Software Developer Intern (Enterprise Applications)</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
@@ -8959,17 +8955,17 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>Hewlett Packard (HP)</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Associate C++ Software Developer</t>
+          <t>Software Engineering Intern/ Co-op</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
@@ -8980,7 +8976,7 @@
       <c r="E294" s="4" t="inlineStr"/>
       <c r="F294" s="4" t="inlineStr">
         <is>
-          <t>Sep 15</t>
+          <t>Sep 18</t>
         </is>
       </c>
     </row>
@@ -9015,17 +9011,17 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Hewlett Packard (HP)</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Intern – Software Developer</t>
+          <t>Associate C++ Software Developer</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
@@ -9036,24 +9032,24 @@
       <c r="E296" s="4" t="inlineStr"/>
       <c r="F296" s="4" t="inlineStr">
         <is>
-          <t>Sep 10</t>
+          <t>Sep 15</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>Arc'teryx Equipment</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Student</t>
+          <t>Intern – Software Developer</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote in Canada</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
@@ -9064,24 +9060,24 @@
       <c r="E297" s="4" t="inlineStr"/>
       <c r="F297" s="4" t="inlineStr">
         <is>
-          <t>Sep 08</t>
+          <t>Sep 10</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Arc'teryx Equipment</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer Co-op Student</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
@@ -9092,24 +9088,24 @@
       <c r="E298" s="4" t="inlineStr"/>
       <c r="F298" s="4" t="inlineStr">
         <is>
-          <t>Sep 05</t>
+          <t>Sep 08</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer: Internship Opportunities</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -9120,19 +9116,19 @@
       <c r="E299" s="4" t="inlineStr"/>
       <c r="F299" s="4" t="inlineStr">
         <is>
-          <t>Sep 5</t>
+          <t>Sep 05</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>Epic Games</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce Programmer Intern</t>
+          <t>Software Engineer: Internship Opportunities</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
@@ -9148,19 +9144,19 @@
       <c r="E300" s="4" t="inlineStr"/>
       <c r="F300" s="4" t="inlineStr">
         <is>
-          <t>Sep 04</t>
+          <t>Sep 5</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Epic Games</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Ecommerce Programmer Intern</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
@@ -9176,24 +9172,24 @@
       <c r="E301" s="4" t="inlineStr"/>
       <c r="F301" s="4" t="inlineStr">
         <is>
-          <t>Sep 01</t>
+          <t>Sep 04</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC Energy</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Computer Science Interns</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
@@ -9204,24 +9200,24 @@
       <c r="E302" s="4" t="inlineStr"/>
       <c r="F302" s="4" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 01</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>Corpay</t>
+          <t>TC Energy</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Software Developer (Co-op)</t>
+          <t>Computer Science Interns</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
@@ -9232,24 +9228,24 @@
       <c r="E303" s="4" t="inlineStr"/>
       <c r="F303" s="4" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Aug 31</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>Dropbox</t>
+          <t>Corpay</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer (Co-op)</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Remote in Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
@@ -9260,19 +9256,19 @@
       <c r="E304" s="4" t="inlineStr"/>
       <c r="F304" s="4" t="inlineStr">
         <is>
-          <t>Aug 25</t>
+          <t>Aug 27</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>Jonas Software</t>
+          <t>Dropbox</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Jonas Summer Internship – Various Departments</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
@@ -9288,12 +9284,40 @@
       <c r="E305" s="4" t="inlineStr"/>
       <c r="F305" s="4" t="inlineStr">
         <is>
+          <t>Aug 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Software</t>
+        </is>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>Jonas Summer Internship – Various Departments</t>
+        </is>
+      </c>
+      <c r="C306" s="4" t="inlineStr">
+        <is>
+          <t>Remote in Canada</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr"/>
+      <c r="F306" s="4" t="inlineStr">
+        <is>
           <t>Aug 02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F305"/>
+  <autoFilter ref="A1:F306"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-08-30
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Investment Management Intern, Canadian Equities</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Aug 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Data Analyst Co-op</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
+          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Ontario-Remote-Work/Data-Analyst-Co-Op_R67175</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Cloud, Data and AI Intern</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -611,17 +611,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Cloud, Data and AI Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Fort-McMurray-Base-Plant-AB-CAN/Automation--Software-or-Computer-Engineering-Student---January-2027_R0017525</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Summer Intern, SAP</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Calgary-AB-CAN/Data-Science-Student---January-2027_R0017534</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Suncor</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20508</t>
+          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Fort-McMurray-Base-Plant-AB-CAN/Automation--Software-or-Computer-Engineering-Student---January-2027_R0017525</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Aug 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Suncor</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Data Science Student</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,117 +727,125 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556956276</t>
+          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Calgary-AB-CAN/Data-Science-Student---January-2027_R0017534</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Aug 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20508</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556956276</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Onware</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Full Stack Developer, Intern</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Edmonton, AB</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Jul 21, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Aug 2, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>British Columbia Investment</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Victoria, BC</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>May 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>CLEAResult</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Energy Efficiency Analyst Co-op</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -848,24 +856,24 @@
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -876,12 +884,96 @@
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="4" t="inlineStr">
         <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F13"/>
+  <autoFilter ref="A1:F16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-09-06
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -547,17 +547,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst Co-op</t>
+          <t>Cloud, Data and AI Intern</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Ontario-Remote-Work/Data-Analyst-Co-Op_R67175</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -616,12 +616,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Summer Intern, SAP</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -643,17 +643,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Suncor</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
+          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Fort-McMurray-Base-Plant-AB-CAN/Automation--Software-or-Computer-Engineering-Student---January-2027_R0017525</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Aug 17, 2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Data Science Student</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Fort-McMurray-Base-Plant-AB-CAN/Automation--Software-or-Computer-Engineering-Student---January-2027_R0017525</t>
+          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Calgary-AB-CAN/Data-Science-Student---January-2027_R0017534</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -707,17 +707,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Engineering Co-op, Electric Division</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Calgary-AB-CAN/Data-Science-Student---January-2027_R0017534</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20508</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Aug 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Software Engineer Intern, Gears of War</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,29 +759,29 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20508</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556956276</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Aug 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Onware</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Full Stack Developer, Intern</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,44 +791,40 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556956276</t>
+          <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Jul 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Onware</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Full Stack Developer, Intern</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Edmonton, AB</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Jul 21, 2026</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Motorola</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Data Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>